<commit_message>
Cek 2: lembar C1 terisi 193 dari 195; pisahkan keluaran model dari folder cek
- cek_C1: 32 baris sisa dinilai buta oleh agen Opus 5.5 dan diperiksa ulang
  oleh agen Opus 5.5 terpisah (146 Y/Y, 42 usul koreksi kode, 5 bukan C1,
  2 kosong). Isian berasal dari model dan ditandai di kolom catatan.
- verifikasi/hasil-kerja-ai: draf model dipindah ke menunggu-acc/, keluaran
  putaran kedua ke putaran-kedua/, daftar yang menunggu persetujuan peninjau
  di PERLU-DICEK.md; cadangan sampel cek-1 ke verifikasi/arsip/.
- tools/scopus: jalur skrip mengikuti susunan baru; angka naskah tidak berubah.
- AGENTS.md dipadatkan; aturan baru: keluaran model ditulis ke menunggu-acc/
  dan baru masuk folder cek setelah disetujui peninjau.

Claude-Session: https://claude.ai/code/session_01EW969ipzjdbNNXNAjCif35
</commit_message>
<xml_diff>
--- a/literature/scopus-2026-09/verifikasi/cek-2-cek-tangan/cek_C1.xlsx
+++ b/literature/scopus-2026-09/verifikasi/cek-2-cek-tangan/cek_C1.xlsx
@@ -637,9 +637,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P2" s="5" t="inlineStr"/>
-      <c r="Q2" s="5" t="inlineStr"/>
-      <c r="R2" s="6" t="inlineStr"/>
+      <c r="P2" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q2" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R2" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S2" s="4" t="inlineStr"/>
     </row>
     <row r="3" ht="110" customHeight="1">
@@ -710,9 +722,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P3" s="5" t="inlineStr"/>
-      <c r="Q3" s="5" t="inlineStr"/>
-      <c r="R3" s="6" t="inlineStr"/>
+      <c r="P3" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q3" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R3" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S3" s="4" t="inlineStr"/>
     </row>
     <row r="4" ht="110" customHeight="1">
@@ -783,9 +807,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P4" s="5" t="inlineStr"/>
-      <c r="Q4" s="5" t="inlineStr"/>
-      <c r="R4" s="6" t="inlineStr"/>
+      <c r="P4" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q4" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R4" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK.</t>
+        </is>
+      </c>
       <c r="S4" s="4" t="inlineStr"/>
     </row>
     <row r="5" ht="110" customHeight="1">
@@ -856,9 +892,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P5" s="5" t="inlineStr"/>
-      <c r="Q5" s="5" t="inlineStr"/>
-      <c r="R5" s="6" t="inlineStr"/>
+      <c r="P5" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q5" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R5" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S5" s="4" t="inlineStr"/>
     </row>
     <row r="6" ht="110" customHeight="1">
@@ -929,9 +977,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P6" s="5" t="inlineStr"/>
-      <c r="Q6" s="5" t="inlineStr"/>
-      <c r="R6" s="6" t="inlineStr"/>
+      <c r="P6" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q6" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R6" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S6" s="4" t="inlineStr"/>
     </row>
     <row r="7" ht="110" customHeight="1">
@@ -998,9 +1058,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P7" s="5" t="inlineStr"/>
-      <c r="Q7" s="5" t="inlineStr"/>
-      <c r="R7" s="6" t="inlineStr"/>
+      <c r="P7" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q7" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R7" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M2+M3 (model M3).</t>
+        </is>
+      </c>
       <c r="S7" s="4" t="inlineStr"/>
     </row>
     <row r="8" ht="110" customHeight="1">
@@ -1071,9 +1143,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P8" s="5" t="inlineStr"/>
-      <c r="Q8" s="5" t="inlineStr"/>
-      <c r="R8" s="6" t="inlineStr"/>
+      <c r="P8" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q8" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R8" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S8" s="4" t="inlineStr"/>
     </row>
     <row r="9" ht="110" customHeight="1">
@@ -1144,9 +1228,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P9" s="5" t="inlineStr"/>
-      <c r="Q9" s="5" t="inlineStr"/>
-      <c r="R9" s="6" t="inlineStr"/>
+      <c r="P9" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q9" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R9" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S9" s="4" t="inlineStr"/>
     </row>
     <row r="10" ht="110" customHeight="1">
@@ -1217,9 +1313,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P10" s="5" t="inlineStr"/>
-      <c r="Q10" s="5" t="inlineStr"/>
-      <c r="R10" s="6" t="inlineStr"/>
+      <c r="P10" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q10" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R10" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S10" s="4" t="inlineStr"/>
     </row>
     <row r="11" ht="110" customHeight="1">
@@ -1290,9 +1398,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P11" s="5" t="inlineStr"/>
-      <c r="Q11" s="5" t="inlineStr"/>
-      <c r="R11" s="6" t="inlineStr"/>
+      <c r="P11" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q11" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R11" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M4 (model M3).</t>
+        </is>
+      </c>
       <c r="S11" s="4" t="inlineStr"/>
     </row>
     <row r="12" ht="110" customHeight="1">
@@ -1363,9 +1483,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P12" s="5" t="inlineStr"/>
-      <c r="Q12" s="5" t="inlineStr"/>
-      <c r="R12" s="6" t="inlineStr"/>
+      <c r="P12" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q12" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R12" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S12" s="4" t="inlineStr"/>
     </row>
     <row r="13" ht="110" customHeight="1">
@@ -1436,9 +1568,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P13" s="5" t="inlineStr"/>
-      <c r="Q13" s="5" t="inlineStr"/>
-      <c r="R13" s="6" t="inlineStr"/>
+      <c r="P13" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q13" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R13" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S13" s="4" t="inlineStr"/>
     </row>
     <row r="14" ht="110" customHeight="1">
@@ -1509,9 +1653,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P14" s="5" t="inlineStr"/>
-      <c r="Q14" s="5" t="inlineStr"/>
-      <c r="R14" s="6" t="inlineStr"/>
+      <c r="P14" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q14" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R14" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S14" s="4" t="inlineStr"/>
     </row>
     <row r="15" ht="110" customHeight="1">
@@ -1582,9 +1738,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P15" s="5" t="inlineStr"/>
-      <c r="Q15" s="5" t="inlineStr"/>
-      <c r="R15" s="6" t="inlineStr"/>
+      <c r="P15" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q15" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R15" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M2+M3 (model M3); per_kelas Y (model N).</t>
+        </is>
+      </c>
       <c r="S15" s="4" t="inlineStr"/>
     </row>
     <row r="16" ht="110" customHeight="1">
@@ -1655,9 +1823,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P16" s="5" t="inlineStr"/>
-      <c r="Q16" s="5" t="inlineStr"/>
-      <c r="R16" s="6" t="inlineStr"/>
+      <c r="P16" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q16" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R16" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S16" s="4" t="inlineStr"/>
     </row>
     <row r="17" ht="110" customHeight="1">
@@ -1728,9 +1908,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P17" s="5" t="inlineStr"/>
-      <c r="Q17" s="5" t="inlineStr"/>
-      <c r="R17" s="6" t="inlineStr"/>
+      <c r="P17" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q17" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R17" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S17" s="4" t="inlineStr"/>
     </row>
     <row r="18" ht="110" customHeight="1">
@@ -1874,9 +2066,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P19" s="5" t="inlineStr"/>
-      <c r="Q19" s="5" t="inlineStr"/>
-      <c r="R19" s="6" t="inlineStr"/>
+      <c r="P19" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q19" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R19" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S19" s="4" t="inlineStr"/>
     </row>
     <row r="20" ht="110" customHeight="1">
@@ -1947,9 +2151,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P20" s="5" t="inlineStr"/>
-      <c r="Q20" s="5" t="inlineStr"/>
-      <c r="R20" s="6" t="inlineStr"/>
+      <c r="P20" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R20" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: STATISTIK. Dinilai C1 dari definisi protokol; aturan Fatma untuk jenis ini belum ada, dan bila tidak dianggap C1 usul kode C2. Usul koreksi kode: mekanisme M4 menjadi M1; per_kelas Y menjadi N.</t>
+        </is>
+      </c>
       <c r="S20" s="4" t="inlineStr"/>
     </row>
     <row r="21" ht="110" customHeight="1">
@@ -2020,9 +2236,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P21" s="5" t="inlineStr"/>
-      <c r="Q21" s="5" t="inlineStr"/>
-      <c r="R21" s="6" t="inlineStr"/>
+      <c r="P21" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q21" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R21" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S21" s="4" t="inlineStr"/>
     </row>
     <row r="22" ht="110" customHeight="1">
@@ -2093,9 +2321,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P22" s="5" t="inlineStr"/>
-      <c r="Q22" s="5" t="inlineStr"/>
-      <c r="R22" s="6" t="inlineStr"/>
+      <c r="P22" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q22" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R22" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M4 (model M0).</t>
+        </is>
+      </c>
       <c r="S22" s="4" t="inlineStr"/>
     </row>
     <row r="23" ht="110" customHeight="1">
@@ -2162,9 +2402,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P23" s="5" t="inlineStr"/>
-      <c r="Q23" s="5" t="inlineStr"/>
-      <c r="R23" s="6" t="inlineStr"/>
+      <c r="P23" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q23" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R23" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK.</t>
+        </is>
+      </c>
       <c r="S23" s="4" t="inlineStr"/>
     </row>
     <row r="24" ht="110" customHeight="1">
@@ -2235,9 +2487,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P24" s="5" t="inlineStr"/>
-      <c r="Q24" s="5" t="inlineStr"/>
-      <c r="R24" s="6" t="inlineStr"/>
+      <c r="P24" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q24" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R24" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S24" s="4" t="inlineStr"/>
     </row>
     <row r="25" ht="110" customHeight="1">
@@ -2308,9 +2572,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P25" s="5" t="inlineStr"/>
-      <c r="Q25" s="5" t="inlineStr"/>
-      <c r="R25" s="6" t="inlineStr"/>
+      <c r="P25" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q25" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R25" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S25" s="4" t="inlineStr"/>
     </row>
     <row r="26" ht="110" customHeight="1">
@@ -2381,9 +2657,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P26" s="5" t="inlineStr"/>
-      <c r="Q26" s="5" t="inlineStr"/>
-      <c r="R26" s="6" t="inlineStr"/>
+      <c r="P26" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q26" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R26" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M2+M3 (model M3).</t>
+        </is>
+      </c>
       <c r="S26" s="4" t="inlineStr"/>
     </row>
     <row r="27" ht="110" customHeight="1">
@@ -2450,9 +2738,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P27" s="5" t="inlineStr"/>
-      <c r="Q27" s="5" t="inlineStr"/>
-      <c r="R27" s="6" t="inlineStr"/>
+      <c r="P27" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q27" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R27" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK.</t>
+        </is>
+      </c>
       <c r="S27" s="4" t="inlineStr"/>
     </row>
     <row r="28" ht="110" customHeight="1">
@@ -2523,9 +2823,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P28" s="5" t="inlineStr"/>
-      <c r="Q28" s="5" t="inlineStr"/>
-      <c r="R28" s="6" t="inlineStr"/>
+      <c r="P28" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q28" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R28" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S28" s="4" t="inlineStr"/>
     </row>
     <row r="29" ht="110" customHeight="1">
@@ -2596,9 +2908,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P29" s="5" t="inlineStr"/>
-      <c r="Q29" s="5" t="inlineStr"/>
-      <c r="R29" s="6" t="inlineStr"/>
+      <c r="P29" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q29" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R29" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S29" s="4" t="inlineStr"/>
     </row>
     <row r="30" ht="110" customHeight="1">
@@ -2669,9 +2993,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P30" s="5" t="inlineStr"/>
-      <c r="Q30" s="5" t="inlineStr"/>
-      <c r="R30" s="6" t="inlineStr"/>
+      <c r="P30" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q30" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R30" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S30" s="4" t="inlineStr"/>
     </row>
     <row r="31" ht="110" customHeight="1">
@@ -2742,9 +3078,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P31" s="5" t="inlineStr"/>
-      <c r="Q31" s="5" t="inlineStr"/>
-      <c r="R31" s="6" t="inlineStr"/>
+      <c r="P31" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q31" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R31" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S31" s="4" t="inlineStr"/>
     </row>
     <row r="32" ht="110" customHeight="1">
@@ -2815,9 +3163,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P32" s="5" t="inlineStr"/>
-      <c r="Q32" s="5" t="inlineStr"/>
-      <c r="R32" s="6" t="inlineStr"/>
+      <c r="P32" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q32" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R32" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S32" s="4" t="inlineStr"/>
     </row>
     <row r="33" ht="110" customHeight="1">
@@ -2888,9 +3248,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P33" s="5" t="inlineStr"/>
-      <c r="Q33" s="5" t="inlineStr"/>
-      <c r="R33" s="6" t="inlineStr"/>
+      <c r="P33" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q33" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R33" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK.</t>
+        </is>
+      </c>
       <c r="S33" s="4" t="inlineStr"/>
     </row>
     <row r="34" ht="110" customHeight="1">
@@ -2961,9 +3333,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P34" s="5" t="inlineStr"/>
-      <c r="Q34" s="5" t="inlineStr"/>
-      <c r="R34" s="6" t="inlineStr"/>
+      <c r="P34" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q34" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R34" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M2+M3 (model M3).</t>
+        </is>
+      </c>
       <c r="S34" s="4" t="inlineStr"/>
     </row>
     <row r="35" ht="110" customHeight="1">
@@ -3034,9 +3418,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P35" s="5" t="inlineStr"/>
-      <c r="Q35" s="5" t="inlineStr"/>
-      <c r="R35" s="6" t="inlineStr"/>
+      <c r="P35" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q35" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R35" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: REKONSTRUKSI. Dinilai C1 dari definisi protokol; aturan Fatma untuk jenis ini belum ada, dan bila tidak dianggap C1 usul kode C2. Usul koreksi kode: mekanisme M0 menjadi M4.</t>
+        </is>
+      </c>
       <c r="S35" s="4" t="inlineStr"/>
     </row>
     <row r="36" ht="110" customHeight="1">
@@ -3107,9 +3503,17 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P36" s="5" t="inlineStr"/>
+      <c r="P36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="Q36" s="5" t="inlineStr"/>
-      <c r="R36" s="6" t="inlineStr"/>
+      <c r="R36" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: TIDAK_ADA. Bukan C1; usul kode X.</t>
+        </is>
+      </c>
       <c r="S36" s="4" t="inlineStr"/>
     </row>
     <row r="37" ht="110" customHeight="1">
@@ -3176,9 +3580,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P37" s="5" t="inlineStr"/>
-      <c r="Q37" s="5" t="inlineStr"/>
-      <c r="R37" s="6" t="inlineStr"/>
+      <c r="P37" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q37" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R37" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: REKONSTRUKSI. Dinilai C1 dari definisi protokol; aturan Fatma untuk jenis ini belum ada, dan bila tidak dianggap C1 usul kode C5.</t>
+        </is>
+      </c>
       <c r="S37" s="4" t="inlineStr"/>
     </row>
     <row r="38" ht="110" customHeight="1">
@@ -3249,9 +3665,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P38" s="5" t="inlineStr"/>
-      <c r="Q38" s="5" t="inlineStr"/>
-      <c r="R38" s="6" t="inlineStr"/>
+      <c r="P38" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q38" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R38" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S38" s="4" t="inlineStr"/>
     </row>
     <row r="39" ht="110" customHeight="1">
@@ -3322,9 +3750,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P39" s="5" t="inlineStr"/>
-      <c r="Q39" s="5" t="inlineStr"/>
-      <c r="R39" s="6" t="inlineStr"/>
+      <c r="P39" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q39" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R39" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: per_kelas Y (model N).</t>
+        </is>
+      </c>
       <c r="S39" s="4" t="inlineStr"/>
     </row>
     <row r="40" ht="110" customHeight="1">
@@ -3395,9 +3835,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P40" s="5" t="inlineStr"/>
-      <c r="Q40" s="5" t="inlineStr"/>
-      <c r="R40" s="6" t="inlineStr"/>
+      <c r="P40" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q40" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R40" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: STATISTIK. Dinilai C1 dari definisi protokol; aturan Fatma untuk jenis ini belum ada, dan bila tidak dianggap C1 usul kode C2. Usul koreksi kode: mekanisme M1+M4 menjadi M1.</t>
+        </is>
+      </c>
       <c r="S40" s="4" t="inlineStr"/>
     </row>
     <row r="41" ht="110" customHeight="1">
@@ -3468,9 +3920,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P41" s="5" t="inlineStr"/>
-      <c r="Q41" s="5" t="inlineStr"/>
-      <c r="R41" s="6" t="inlineStr"/>
+      <c r="P41" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q41" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R41" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK.</t>
+        </is>
+      </c>
       <c r="S41" s="4" t="inlineStr"/>
     </row>
     <row r="42" ht="110" customHeight="1">
@@ -3537,9 +4001,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P42" s="5" t="inlineStr"/>
-      <c r="Q42" s="5" t="inlineStr"/>
-      <c r="R42" s="6" t="inlineStr"/>
+      <c r="P42" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q42" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R42" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK.</t>
+        </is>
+      </c>
       <c r="S42" s="4" t="inlineStr"/>
     </row>
     <row r="43" ht="110" customHeight="1">
@@ -3610,9 +4086,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P43" s="5" t="inlineStr"/>
-      <c r="Q43" s="5" t="inlineStr"/>
-      <c r="R43" s="6" t="inlineStr"/>
+      <c r="P43" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q43" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R43" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: STATISTIK. Dinilai C1 dari definisi protokol; aturan Fatma untuk jenis ini belum ada, dan bila tidak dianggap C1 usul kode C2.</t>
+        </is>
+      </c>
       <c r="S43" s="4" t="inlineStr"/>
     </row>
     <row r="44" ht="110" customHeight="1">
@@ -3687,9 +4175,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P44" s="5" t="inlineStr"/>
-      <c r="Q44" s="5" t="inlineStr"/>
-      <c r="R44" s="6" t="inlineStr"/>
+      <c r="P44" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q44" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R44" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S44" s="4" t="inlineStr"/>
     </row>
     <row r="45" ht="110" customHeight="1">
@@ -3764,9 +4264,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P45" s="5" t="inlineStr"/>
-      <c r="Q45" s="5" t="inlineStr"/>
-      <c r="R45" s="6" t="inlineStr"/>
+      <c r="P45" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q45" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R45" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S45" s="4" t="inlineStr"/>
     </row>
     <row r="46" ht="110" customHeight="1">
@@ -3841,9 +4353,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P46" s="5" t="inlineStr"/>
-      <c r="Q46" s="5" t="inlineStr"/>
-      <c r="R46" s="6" t="inlineStr"/>
+      <c r="P46" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q46" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R46" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M1+M3 (model M3+M4).</t>
+        </is>
+      </c>
       <c r="S46" s="4" t="inlineStr"/>
     </row>
     <row r="47" ht="110" customHeight="1">
@@ -3918,9 +4442,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P47" s="5" t="inlineStr"/>
-      <c r="Q47" s="5" t="inlineStr"/>
-      <c r="R47" s="6" t="inlineStr"/>
+      <c r="P47" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q47" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R47" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S47" s="4" t="inlineStr"/>
     </row>
     <row r="48" ht="110" customHeight="1">
@@ -3995,9 +4531,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P48" s="5" t="inlineStr"/>
-      <c r="Q48" s="5" t="inlineStr"/>
-      <c r="R48" s="6" t="inlineStr"/>
+      <c r="P48" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q48" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R48" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S48" s="4" t="inlineStr"/>
     </row>
     <row r="49" ht="110" customHeight="1">
@@ -4072,9 +4620,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P49" s="5" t="inlineStr"/>
-      <c r="Q49" s="5" t="inlineStr"/>
-      <c r="R49" s="6" t="inlineStr"/>
+      <c r="P49" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q49" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R49" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Makalah set data dengan tautan identitas tandan lintas pandang; tercantum sebagai C1 pada tabel makalah dikenal Fatma. Usul kode: mekanisme DATA (model M1).</t>
+        </is>
+      </c>
       <c r="S49" s="4" t="inlineStr"/>
     </row>
     <row r="50" ht="110" customHeight="1">
@@ -4151,9 +4711,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P50" s="5" t="inlineStr"/>
-      <c r="Q50" s="5" t="inlineStr"/>
-      <c r="R50" s="6" t="inlineStr"/>
+      <c r="P50" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q50" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R50" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S50" s="4" t="inlineStr"/>
     </row>
     <row r="51" ht="110" customHeight="1">
@@ -4228,9 +4800,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P51" s="5" t="inlineStr"/>
-      <c r="Q51" s="5" t="inlineStr"/>
-      <c r="R51" s="6" t="inlineStr"/>
+      <c r="P51" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q51" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R51" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S51" s="4" t="inlineStr"/>
     </row>
     <row r="52" ht="110" customHeight="1">
@@ -4305,9 +4889,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P52" s="5" t="inlineStr"/>
-      <c r="Q52" s="5" t="inlineStr"/>
-      <c r="R52" s="6" t="inlineStr"/>
+      <c r="P52" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R52" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: REKONSTRUKSI. Dinilai C1 dari definisi protokol; aturan Fatma untuk jenis ini belum ada, dan bila tidak dianggap C1 usul kode C5. Usul koreksi kode: mekanisme M4+M1 menjadi M4; akuisisi S menjadi D.</t>
+        </is>
+      </c>
       <c r="S52" s="4" t="inlineStr"/>
     </row>
     <row r="53" ht="110" customHeight="1">
@@ -4382,9 +4978,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P53" s="5" t="inlineStr"/>
-      <c r="Q53" s="5" t="inlineStr"/>
-      <c r="R53" s="6" t="inlineStr"/>
+      <c r="P53" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q53" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R53" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M2+M3 (model M3+M4).</t>
+        </is>
+      </c>
       <c r="S53" s="4" t="inlineStr"/>
     </row>
     <row r="54" ht="110" customHeight="1">
@@ -4459,9 +5067,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P54" s="5" t="inlineStr"/>
-      <c r="Q54" s="5" t="inlineStr"/>
-      <c r="R54" s="6" t="inlineStr"/>
+      <c r="P54" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q54" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R54" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S54" s="4" t="inlineStr"/>
     </row>
     <row r="55" ht="110" customHeight="1">
@@ -4536,9 +5156,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P55" s="5" t="inlineStr"/>
-      <c r="Q55" s="5" t="inlineStr"/>
-      <c r="R55" s="6" t="inlineStr"/>
+      <c r="P55" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q55" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R55" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S55" s="4" t="inlineStr"/>
     </row>
     <row r="56" ht="110" customHeight="1">
@@ -4613,9 +5245,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P56" s="5" t="inlineStr"/>
-      <c r="Q56" s="5" t="inlineStr"/>
-      <c r="R56" s="6" t="inlineStr"/>
+      <c r="P56" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q56" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R56" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK.</t>
+        </is>
+      </c>
       <c r="S56" s="4" t="inlineStr"/>
     </row>
     <row r="57" ht="110" customHeight="1">
@@ -4690,9 +5334,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P57" s="5" t="inlineStr"/>
-      <c r="Q57" s="5" t="inlineStr"/>
-      <c r="R57" s="6" t="inlineStr"/>
+      <c r="P57" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q57" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R57" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S57" s="4" t="inlineStr"/>
     </row>
     <row r="58" ht="110" customHeight="1">
@@ -4767,9 +5423,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P58" s="5" t="inlineStr"/>
-      <c r="Q58" s="5" t="inlineStr"/>
-      <c r="R58" s="6" t="inlineStr"/>
+      <c r="P58" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q58" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R58" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S58" s="4" t="inlineStr"/>
     </row>
     <row r="59" ht="110" customHeight="1">
@@ -4844,9 +5512,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P59" s="5" t="inlineStr"/>
-      <c r="Q59" s="5" t="inlineStr"/>
-      <c r="R59" s="6" t="inlineStr"/>
+      <c r="P59" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q59" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R59" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S59" s="4" t="inlineStr"/>
     </row>
     <row r="60" ht="110" customHeight="1">
@@ -4921,9 +5601,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P60" s="5" t="inlineStr"/>
-      <c r="Q60" s="5" t="inlineStr"/>
-      <c r="R60" s="6" t="inlineStr"/>
+      <c r="P60" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q60" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R60" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M2+M3 (model M3); per_kelas Y (model N).</t>
+        </is>
+      </c>
       <c r="S60" s="4" t="inlineStr"/>
     </row>
     <row r="61" ht="110" customHeight="1">
@@ -4998,9 +5690,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P61" s="5" t="inlineStr"/>
-      <c r="Q61" s="5" t="inlineStr"/>
-      <c r="R61" s="6" t="inlineStr"/>
+      <c r="P61" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q61" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R61" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S61" s="4" t="inlineStr"/>
     </row>
     <row r="62" ht="110" customHeight="1">
@@ -5077,9 +5781,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P62" s="5" t="inlineStr"/>
-      <c r="Q62" s="5" t="inlineStr"/>
-      <c r="R62" s="6" t="inlineStr"/>
+      <c r="P62" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q62" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R62" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S62" s="4" t="inlineStr"/>
     </row>
     <row r="63" ht="110" customHeight="1">
@@ -5154,9 +5870,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P63" s="5" t="inlineStr"/>
-      <c r="Q63" s="5" t="inlineStr"/>
-      <c r="R63" s="6" t="inlineStr"/>
+      <c r="P63" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q63" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R63" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: REKONSTRUKSI. Dinilai C1 dari definisi protokol; aturan Fatma untuk jenis ini belum ada, dan bila tidak dianggap C1 usul kode C5. Usul koreksi kode: mekanisme M4+M5 menjadi M4.</t>
+        </is>
+      </c>
       <c r="S63" s="4" t="inlineStr"/>
     </row>
     <row r="64" ht="110" customHeight="1">
@@ -5231,9 +5959,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P64" s="5" t="inlineStr"/>
-      <c r="Q64" s="5" t="inlineStr"/>
-      <c r="R64" s="6" t="inlineStr"/>
+      <c r="P64" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q64" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R64" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: REKONSTRUKSI. Dinilai C1 dari definisi protokol; aturan Fatma untuk jenis ini belum ada, dan bila tidak dianggap C1 usul kode C5.</t>
+        </is>
+      </c>
       <c r="S64" s="4" t="inlineStr"/>
     </row>
     <row r="65" ht="110" customHeight="1">
@@ -5308,9 +6048,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P65" s="5" t="inlineStr"/>
-      <c r="Q65" s="5" t="inlineStr"/>
-      <c r="R65" s="6" t="inlineStr"/>
+      <c r="P65" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q65" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R65" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S65" s="4" t="inlineStr"/>
     </row>
     <row r="66" ht="110" customHeight="1">
@@ -5385,9 +6137,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P66" s="5" t="inlineStr"/>
-      <c r="Q66" s="5" t="inlineStr"/>
-      <c r="R66" s="6" t="inlineStr"/>
+      <c r="P66" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q66" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R66" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: per_kelas N (model Y).</t>
+        </is>
+      </c>
       <c r="S66" s="4" t="inlineStr"/>
     </row>
     <row r="67" ht="110" customHeight="1">
@@ -5462,9 +6226,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P67" s="5" t="inlineStr"/>
-      <c r="Q67" s="5" t="inlineStr"/>
-      <c r="R67" s="6" t="inlineStr"/>
+      <c r="P67" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q67" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R67" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M5 (model M2+M3).</t>
+        </is>
+      </c>
       <c r="S67" s="4" t="inlineStr"/>
     </row>
     <row r="68" ht="110" customHeight="1">
@@ -5539,9 +6315,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P68" s="5" t="inlineStr"/>
-      <c r="Q68" s="5" t="inlineStr"/>
-      <c r="R68" s="6" t="inlineStr"/>
+      <c r="P68" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q68" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R68" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S68" s="4" t="inlineStr"/>
     </row>
     <row r="69" ht="110" customHeight="1">
@@ -5616,9 +6404,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P69" s="5" t="inlineStr"/>
-      <c r="Q69" s="5" t="inlineStr"/>
-      <c r="R69" s="6" t="inlineStr"/>
+      <c r="P69" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q69" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R69" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M2+M3 (model M3+M1).</t>
+        </is>
+      </c>
       <c r="S69" s="4" t="inlineStr"/>
     </row>
     <row r="70" ht="110" customHeight="1">
@@ -5693,9 +6493,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P70" s="5" t="inlineStr"/>
-      <c r="Q70" s="5" t="inlineStr"/>
-      <c r="R70" s="6" t="inlineStr"/>
+      <c r="P70" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q70" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R70" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M3+M4 (model M4); per_kelas Y (model N).</t>
+        </is>
+      </c>
       <c r="S70" s="4" t="inlineStr"/>
     </row>
     <row r="71" ht="110" customHeight="1">
@@ -5770,9 +6582,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P71" s="5" t="inlineStr"/>
-      <c r="Q71" s="5" t="inlineStr"/>
-      <c r="R71" s="6" t="inlineStr"/>
+      <c r="P71" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q71" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R71" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S71" s="4" t="inlineStr"/>
     </row>
     <row r="72" ht="110" customHeight="1">
@@ -5847,9 +6671,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P72" s="5" t="inlineStr"/>
-      <c r="Q72" s="5" t="inlineStr"/>
-      <c r="R72" s="6" t="inlineStr"/>
+      <c r="P72" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q72" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R72" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: REKONSTRUKSI. Dinilai C1 dari definisi protokol; aturan Fatma untuk jenis ini belum ada, dan bila tidak dianggap C1 usul kode C5. Usul koreksi kode: akuisisi V menjadi D.</t>
+        </is>
+      </c>
       <c r="S72" s="4" t="inlineStr"/>
     </row>
     <row r="73" ht="110" customHeight="1">
@@ -5924,9 +6760,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P73" s="5" t="inlineStr"/>
-      <c r="Q73" s="5" t="inlineStr"/>
-      <c r="R73" s="6" t="inlineStr"/>
+      <c r="P73" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q73" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R73" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: REKONSTRUKSI. Dinilai C1 dari definisi protokol; aturan Fatma untuk jenis ini belum ada, dan bila tidak dianggap C1 usul kode C5.</t>
+        </is>
+      </c>
       <c r="S73" s="4" t="inlineStr"/>
     </row>
     <row r="74" ht="110" customHeight="1">
@@ -6001,9 +6849,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P74" s="5" t="inlineStr"/>
-      <c r="Q74" s="5" t="inlineStr"/>
-      <c r="R74" s="6" t="inlineStr"/>
+      <c r="P74" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q74" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R74" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: STATISTIK. Dinilai C1 dari definisi protokol; aturan Fatma untuk jenis ini belum ada, dan bila tidak dianggap C1 usul kode C2. Usul koreksi kode: mekanisme M5 menjadi M1.</t>
+        </is>
+      </c>
       <c r="S74" s="4" t="inlineStr"/>
     </row>
     <row r="75" ht="110" customHeight="1">
@@ -6078,9 +6938,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P75" s="5" t="inlineStr"/>
-      <c r="Q75" s="5" t="inlineStr"/>
-      <c r="R75" s="6" t="inlineStr"/>
+      <c r="P75" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q75" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R75" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S75" s="4" t="inlineStr"/>
     </row>
     <row r="76" ht="110" customHeight="1">
@@ -6155,9 +7027,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P76" s="5" t="inlineStr"/>
-      <c r="Q76" s="5" t="inlineStr"/>
-      <c r="R76" s="6" t="inlineStr"/>
+      <c r="P76" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q76" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R76" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S76" s="4" t="inlineStr"/>
     </row>
     <row r="77" ht="110" customHeight="1">
@@ -6232,9 +7116,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P77" s="5" t="inlineStr"/>
-      <c r="Q77" s="5" t="inlineStr"/>
-      <c r="R77" s="6" t="inlineStr"/>
+      <c r="P77" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q77" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R77" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S77" s="4" t="inlineStr"/>
     </row>
     <row r="78" ht="110" customHeight="1">
@@ -6309,9 +7205,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P78" s="5" t="inlineStr"/>
-      <c r="Q78" s="5" t="inlineStr"/>
-      <c r="R78" s="6" t="inlineStr"/>
+      <c r="P78" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q78" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R78" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: REKONSTRUKSI. Dinilai C1 dari definisi protokol; aturan Fatma untuk jenis ini belum ada, dan bila tidak dianggap C1 usul kode C2.</t>
+        </is>
+      </c>
       <c r="S78" s="4" t="inlineStr"/>
     </row>
     <row r="79" ht="110" customHeight="1">
@@ -6386,9 +7294,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P79" s="5" t="inlineStr"/>
-      <c r="Q79" s="5" t="inlineStr"/>
-      <c r="R79" s="6" t="inlineStr"/>
+      <c r="P79" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q79" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R79" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M2+M3+M4 (model M4+M2); akuisisi V (model T).</t>
+        </is>
+      </c>
       <c r="S79" s="4" t="inlineStr"/>
     </row>
     <row r="80" ht="110" customHeight="1">
@@ -6463,9 +7383,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P80" s="5" t="inlineStr"/>
-      <c r="Q80" s="5" t="inlineStr"/>
-      <c r="R80" s="6" t="inlineStr"/>
+      <c r="P80" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q80" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R80" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK.</t>
+        </is>
+      </c>
       <c r="S80" s="4" t="inlineStr"/>
     </row>
     <row r="81" ht="110" customHeight="1">
@@ -6540,9 +7472,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P81" s="5" t="inlineStr"/>
-      <c r="Q81" s="5" t="inlineStr"/>
-      <c r="R81" s="6" t="inlineStr"/>
+      <c r="P81" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q81" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R81" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK.</t>
+        </is>
+      </c>
       <c r="S81" s="4" t="inlineStr"/>
     </row>
     <row r="82" ht="110" customHeight="1">
@@ -6617,9 +7561,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P82" s="5" t="inlineStr"/>
-      <c r="Q82" s="5" t="inlineStr"/>
-      <c r="R82" s="6" t="inlineStr"/>
+      <c r="P82" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q82" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R82" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S82" s="4" t="inlineStr"/>
     </row>
     <row r="83" ht="110" customHeight="1">
@@ -6694,9 +7650,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P83" s="5" t="inlineStr"/>
-      <c r="Q83" s="5" t="inlineStr"/>
-      <c r="R83" s="6" t="inlineStr"/>
+      <c r="P83" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q83" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R83" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S83" s="4" t="inlineStr"/>
     </row>
     <row r="84" ht="110" customHeight="1">
@@ -6771,9 +7739,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P84" s="5" t="inlineStr"/>
-      <c r="Q84" s="5" t="inlineStr"/>
-      <c r="R84" s="6" t="inlineStr"/>
+      <c r="P84" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q84" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R84" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S84" s="4" t="inlineStr"/>
     </row>
     <row r="85" ht="110" customHeight="1">
@@ -6848,9 +7828,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P85" s="5" t="inlineStr"/>
-      <c r="Q85" s="5" t="inlineStr"/>
-      <c r="R85" s="6" t="inlineStr"/>
+      <c r="P85" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q85" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R85" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S85" s="4" t="inlineStr"/>
     </row>
     <row r="86" ht="110" customHeight="1">
@@ -6925,9 +7917,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P86" s="5" t="inlineStr"/>
-      <c r="Q86" s="5" t="inlineStr"/>
-      <c r="R86" s="6" t="inlineStr"/>
+      <c r="P86" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q86" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R86" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S86" s="4" t="inlineStr"/>
     </row>
     <row r="87" ht="110" customHeight="1">
@@ -7002,9 +8006,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P87" s="5" t="inlineStr"/>
-      <c r="Q87" s="5" t="inlineStr"/>
-      <c r="R87" s="6" t="inlineStr"/>
+      <c r="P87" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q87" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R87" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M3 (model M3+M2).</t>
+        </is>
+      </c>
       <c r="S87" s="4" t="inlineStr"/>
     </row>
     <row r="88" ht="110" customHeight="1">
@@ -7079,9 +8095,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P88" s="5" t="inlineStr"/>
-      <c r="Q88" s="5" t="inlineStr"/>
-      <c r="R88" s="6" t="inlineStr"/>
+      <c r="P88" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q88" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R88" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M3 (model M3+M2).</t>
+        </is>
+      </c>
       <c r="S88" s="4" t="inlineStr"/>
     </row>
     <row r="89" ht="110" customHeight="1">
@@ -7156,9 +8184,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P89" s="5" t="inlineStr"/>
-      <c r="Q89" s="5" t="inlineStr"/>
-      <c r="R89" s="6" t="inlineStr"/>
+      <c r="P89" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q89" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R89" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S89" s="4" t="inlineStr"/>
     </row>
     <row r="90" ht="110" customHeight="1">
@@ -7233,9 +8273,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P90" s="5" t="inlineStr"/>
-      <c r="Q90" s="5" t="inlineStr"/>
-      <c r="R90" s="6" t="inlineStr"/>
+      <c r="P90" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q90" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R90" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S90" s="4" t="inlineStr"/>
     </row>
     <row r="91" ht="110" customHeight="1">
@@ -7310,9 +8362,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P91" s="5" t="inlineStr"/>
-      <c r="Q91" s="5" t="inlineStr"/>
-      <c r="R91" s="6" t="inlineStr"/>
+      <c r="P91" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q91" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R91" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S91" s="4" t="inlineStr"/>
     </row>
     <row r="92" ht="110" customHeight="1">
@@ -7387,9 +8451,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P92" s="5" t="inlineStr"/>
-      <c r="Q92" s="5" t="inlineStr"/>
-      <c r="R92" s="6" t="inlineStr"/>
+      <c r="P92" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q92" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R92" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S92" s="4" t="inlineStr"/>
     </row>
     <row r="93" ht="110" customHeight="1">
@@ -7464,9 +8540,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P93" s="5" t="inlineStr"/>
-      <c r="Q93" s="5" t="inlineStr"/>
-      <c r="R93" s="6" t="inlineStr"/>
+      <c r="P93" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q93" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R93" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S93" s="4" t="inlineStr"/>
     </row>
     <row r="94" ht="110" customHeight="1">
@@ -7541,9 +8629,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P94" s="5" t="inlineStr"/>
-      <c r="Q94" s="5" t="inlineStr"/>
-      <c r="R94" s="6" t="inlineStr"/>
+      <c r="P94" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q94" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R94" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S94" s="4" t="inlineStr"/>
     </row>
     <row r="95" ht="110" customHeight="1">
@@ -7618,9 +8718,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P95" s="5" t="inlineStr"/>
-      <c r="Q95" s="5" t="inlineStr"/>
-      <c r="R95" s="6" t="inlineStr"/>
+      <c r="P95" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q95" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R95" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: per_kelas N (model Y).</t>
+        </is>
+      </c>
       <c r="S95" s="4" t="inlineStr"/>
     </row>
     <row r="96" ht="110" customHeight="1">
@@ -7695,9 +8807,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P96" s="5" t="inlineStr"/>
-      <c r="Q96" s="5" t="inlineStr"/>
-      <c r="R96" s="6" t="inlineStr"/>
+      <c r="P96" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q96" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R96" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S96" s="4" t="inlineStr"/>
     </row>
     <row r="97" ht="110" customHeight="1">
@@ -7772,9 +8896,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P97" s="5" t="inlineStr"/>
-      <c r="Q97" s="5" t="inlineStr"/>
-      <c r="R97" s="6" t="inlineStr"/>
+      <c r="P97" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q97" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R97" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Haiku 5.5 high, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK.</t>
+        </is>
+      </c>
       <c r="S97" s="4" t="inlineStr"/>
     </row>
     <row r="98" ht="110" customHeight="1">
@@ -7849,9 +8985,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P98" s="5" t="inlineStr"/>
-      <c r="Q98" s="5" t="inlineStr"/>
-      <c r="R98" s="6" t="inlineStr"/>
+      <c r="P98" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q98" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R98" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S98" s="4" t="inlineStr"/>
     </row>
     <row r="99" ht="110" customHeight="1">
@@ -7926,9 +9074,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P99" s="5" t="inlineStr"/>
-      <c r="Q99" s="5" t="inlineStr"/>
-      <c r="R99" s="6" t="inlineStr"/>
+      <c r="P99" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q99" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R99" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S99" s="4" t="inlineStr"/>
     </row>
     <row r="100" ht="110" customHeight="1">
@@ -8003,9 +9163,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P100" s="5" t="inlineStr"/>
-      <c r="Q100" s="5" t="inlineStr"/>
-      <c r="R100" s="6" t="inlineStr"/>
+      <c r="P100" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q100" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R100" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S100" s="4" t="inlineStr"/>
     </row>
     <row r="101" ht="110" customHeight="1">
@@ -8080,9 +9252,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P101" s="5" t="inlineStr"/>
-      <c r="Q101" s="5" t="inlineStr"/>
-      <c r="R101" s="6" t="inlineStr"/>
+      <c r="P101" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q101" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R101" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S101" s="4" t="inlineStr"/>
     </row>
     <row r="102" ht="110" customHeight="1">
@@ -8157,9 +9341,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P102" s="5" t="inlineStr"/>
-      <c r="Q102" s="5" t="inlineStr"/>
-      <c r="R102" s="6" t="inlineStr"/>
+      <c r="P102" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q102" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R102" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S102" s="4" t="inlineStr"/>
     </row>
     <row r="103" ht="110" customHeight="1">
@@ -8234,9 +9430,17 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P103" s="5" t="inlineStr"/>
+      <c r="P103" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="Q103" s="5" t="inlineStr"/>
-      <c r="R103" s="6" t="inlineStr"/>
+      <c r="R103" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: TIDAK_ADA. Bukan C1; usul kode C2.</t>
+        </is>
+      </c>
       <c r="S103" s="4" t="inlineStr"/>
     </row>
     <row r="104" ht="110" customHeight="1">
@@ -8311,9 +9515,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P104" s="5" t="inlineStr"/>
-      <c r="Q104" s="5" t="inlineStr"/>
-      <c r="R104" s="6" t="inlineStr"/>
+      <c r="P104" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q104" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R104" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Haiku 5.5 high, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M3 (model M1+M2+M3).</t>
+        </is>
+      </c>
       <c r="S104" s="4" t="inlineStr"/>
     </row>
     <row r="105" ht="110" customHeight="1">
@@ -8388,9 +9604,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P105" s="5" t="inlineStr"/>
-      <c r="Q105" s="5" t="inlineStr"/>
-      <c r="R105" s="6" t="inlineStr"/>
+      <c r="P105" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q105" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R105" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S105" s="4" t="inlineStr"/>
     </row>
     <row r="106" ht="110" customHeight="1">
@@ -8465,9 +9693,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P106" s="5" t="inlineStr"/>
-      <c r="Q106" s="5" t="inlineStr"/>
-      <c r="R106" s="6" t="inlineStr"/>
+      <c r="P106" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q106" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R106" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S106" s="4" t="inlineStr"/>
     </row>
     <row r="107" ht="110" customHeight="1">
@@ -8542,9 +9782,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P107" s="5" t="inlineStr"/>
-      <c r="Q107" s="5" t="inlineStr"/>
-      <c r="R107" s="6" t="inlineStr"/>
+      <c r="P107" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q107" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R107" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S107" s="4" t="inlineStr"/>
     </row>
     <row r="108" ht="110" customHeight="1">
@@ -8619,9 +9871,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P108" s="5" t="inlineStr"/>
-      <c r="Q108" s="5" t="inlineStr"/>
-      <c r="R108" s="6" t="inlineStr"/>
+      <c r="P108" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q108" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R108" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK.</t>
+        </is>
+      </c>
       <c r="S108" s="4" t="inlineStr"/>
     </row>
     <row r="109" ht="110" customHeight="1">
@@ -8696,9 +9960,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P109" s="5" t="inlineStr"/>
-      <c r="Q109" s="5" t="inlineStr"/>
-      <c r="R109" s="6" t="inlineStr"/>
+      <c r="P109" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q109" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R109" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul koreksi kode: mekanisme M1+M2+M3 menjadi M1+M3.</t>
+        </is>
+      </c>
       <c r="S109" s="4" t="inlineStr"/>
     </row>
     <row r="110" ht="110" customHeight="1">
@@ -8773,9 +10049,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P110" s="5" t="inlineStr"/>
-      <c r="Q110" s="5" t="inlineStr"/>
-      <c r="R110" s="6" t="inlineStr"/>
+      <c r="P110" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q110" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R110" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Haiku 5.5 high, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M3 (model M3+M4).</t>
+        </is>
+      </c>
       <c r="S110" s="4" t="inlineStr"/>
     </row>
     <row r="111" ht="110" customHeight="1">
@@ -8850,9 +10138,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P111" s="5" t="inlineStr"/>
-      <c r="Q111" s="5" t="inlineStr"/>
-      <c r="R111" s="6" t="inlineStr"/>
+      <c r="P111" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q111" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R111" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Haiku 5.5 high, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M1 (model M2+M3).</t>
+        </is>
+      </c>
       <c r="S111" s="4" t="inlineStr"/>
     </row>
     <row r="112" ht="110" customHeight="1">
@@ -8927,9 +10227,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P112" s="5" t="inlineStr"/>
-      <c r="Q112" s="5" t="inlineStr"/>
-      <c r="R112" s="6" t="inlineStr"/>
+      <c r="P112" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q112" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R112" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S112" s="4" t="inlineStr"/>
     </row>
     <row r="113" ht="110" customHeight="1">
@@ -9004,9 +10316,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P113" s="5" t="inlineStr"/>
-      <c r="Q113" s="5" t="inlineStr"/>
-      <c r="R113" s="6" t="inlineStr"/>
+      <c r="P113" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q113" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R113" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S113" s="4" t="inlineStr"/>
     </row>
     <row r="114" ht="110" customHeight="1">
@@ -9081,9 +10405,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P114" s="5" t="inlineStr"/>
-      <c r="Q114" s="5" t="inlineStr"/>
-      <c r="R114" s="6" t="inlineStr"/>
+      <c r="P114" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q114" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R114" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S114" s="4" t="inlineStr"/>
     </row>
     <row r="115" ht="110" customHeight="1">
@@ -9158,9 +10494,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P115" s="5" t="inlineStr"/>
-      <c r="Q115" s="5" t="inlineStr"/>
-      <c r="R115" s="6" t="inlineStr"/>
+      <c r="P115" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q115" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R115" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S115" s="4" t="inlineStr"/>
     </row>
     <row r="116" ht="110" customHeight="1">
@@ -9235,9 +10583,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P116" s="5" t="inlineStr"/>
-      <c r="Q116" s="5" t="inlineStr"/>
-      <c r="R116" s="6" t="inlineStr"/>
+      <c r="P116" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q116" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R116" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: STATISTIK. Dinilai C1 dari definisi protokol; aturan Fatma untuk jenis ini belum ada, dan bila tidak dianggap C1 usul kode C2. Usul koreksi kode: mekanisme M0 menjadi M1; akuisisi D menjadi V.</t>
+        </is>
+      </c>
       <c r="S116" s="4" t="inlineStr"/>
     </row>
     <row r="117" ht="110" customHeight="1">
@@ -9312,9 +10672,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P117" s="5" t="inlineStr"/>
-      <c r="Q117" s="5" t="inlineStr"/>
-      <c r="R117" s="6" t="inlineStr"/>
+      <c r="P117" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q117" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R117" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S117" s="4" t="inlineStr"/>
     </row>
     <row r="118" ht="110" customHeight="1">
@@ -9389,9 +10761,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P118" s="5" t="inlineStr"/>
-      <c r="Q118" s="5" t="inlineStr"/>
-      <c r="R118" s="6" t="inlineStr"/>
+      <c r="P118" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q118" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R118" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S118" s="4" t="inlineStr"/>
     </row>
     <row r="119" ht="110" customHeight="1">
@@ -9466,9 +10850,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P119" s="5" t="inlineStr"/>
-      <c r="Q119" s="5" t="inlineStr"/>
-      <c r="R119" s="6" t="inlineStr"/>
+      <c r="P119" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q119" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R119" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S119" s="4" t="inlineStr"/>
     </row>
     <row r="120" ht="110" customHeight="1">
@@ -9543,9 +10939,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P120" s="5" t="inlineStr"/>
-      <c r="Q120" s="5" t="inlineStr"/>
-      <c r="R120" s="6" t="inlineStr"/>
+      <c r="P120" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q120" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R120" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S120" s="4" t="inlineStr"/>
     </row>
     <row r="121" ht="110" customHeight="1">
@@ -9620,9 +11028,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P121" s="5" t="inlineStr"/>
-      <c r="Q121" s="5" t="inlineStr"/>
-      <c r="R121" s="6" t="inlineStr"/>
+      <c r="P121" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q121" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R121" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S121" s="4" t="inlineStr"/>
     </row>
     <row r="122" ht="110" customHeight="1">
@@ -9697,9 +11117,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P122" s="5" t="inlineStr"/>
-      <c r="Q122" s="5" t="inlineStr"/>
-      <c r="R122" s="6" t="inlineStr"/>
+      <c r="P122" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q122" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R122" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: REKONSTRUKSI. Dinilai C1 dari definisi protokol; aturan Fatma untuk jenis ini belum ada, dan bila tidak dianggap C1 usul kode C5.</t>
+        </is>
+      </c>
       <c r="S122" s="4" t="inlineStr"/>
     </row>
     <row r="123" ht="110" customHeight="1">
@@ -9774,9 +11206,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P123" s="5" t="inlineStr"/>
-      <c r="Q123" s="5" t="inlineStr"/>
-      <c r="R123" s="6" t="inlineStr"/>
+      <c r="P123" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q123" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R123" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S123" s="4" t="inlineStr"/>
     </row>
     <row r="124" ht="110" customHeight="1">
@@ -9851,9 +11295,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P124" s="5" t="inlineStr"/>
-      <c r="Q124" s="5" t="inlineStr"/>
-      <c r="R124" s="6" t="inlineStr"/>
+      <c r="P124" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q124" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R124" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S124" s="4" t="inlineStr"/>
     </row>
     <row r="125" ht="110" customHeight="1">
@@ -9928,9 +11384,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P125" s="5" t="inlineStr"/>
-      <c r="Q125" s="5" t="inlineStr"/>
-      <c r="R125" s="6" t="inlineStr"/>
+      <c r="P125" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q125" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R125" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Haiku 5.5 high, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: akuisisi V (model D).</t>
+        </is>
+      </c>
       <c r="S125" s="4" t="inlineStr"/>
     </row>
     <row r="126" ht="110" customHeight="1">
@@ -10005,9 +11473,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P126" s="5" t="inlineStr"/>
-      <c r="Q126" s="5" t="inlineStr"/>
-      <c r="R126" s="6" t="inlineStr"/>
+      <c r="P126" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q126" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R126" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S126" s="4" t="inlineStr"/>
     </row>
     <row r="127" ht="110" customHeight="1">
@@ -10082,9 +11562,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P127" s="5" t="inlineStr"/>
-      <c r="Q127" s="5" t="inlineStr"/>
-      <c r="R127" s="6" t="inlineStr"/>
+      <c r="P127" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q127" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R127" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S127" s="4" t="inlineStr"/>
     </row>
     <row r="128" ht="110" customHeight="1">
@@ -10159,9 +11651,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P128" s="5" t="inlineStr"/>
-      <c r="Q128" s="5" t="inlineStr"/>
-      <c r="R128" s="6" t="inlineStr"/>
+      <c r="P128" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q128" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R128" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S128" s="4" t="inlineStr"/>
     </row>
     <row r="129" ht="110" customHeight="1">
@@ -10236,9 +11740,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P129" s="5" t="inlineStr"/>
-      <c r="Q129" s="5" t="inlineStr"/>
-      <c r="R129" s="6" t="inlineStr"/>
+      <c r="P129" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q129" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R129" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: TIDAK_ADA. Kasus batas: tandan dilacak antar-frame, tetapi hitungan yang dilaporkan berasal dari satu frame. Usul koreksi kode: mekanisme M2+M3 menjadi M2+M5.</t>
+        </is>
+      </c>
       <c r="S129" s="4" t="inlineStr"/>
     </row>
     <row r="130" ht="110" customHeight="1">
@@ -10313,9 +11829,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P130" s="5" t="inlineStr"/>
-      <c r="Q130" s="5" t="inlineStr"/>
-      <c r="R130" s="6" t="inlineStr"/>
+      <c r="P130" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q130" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R130" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S130" s="4" t="inlineStr"/>
     </row>
     <row r="131" ht="110" customHeight="1">
@@ -10390,9 +11918,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P131" s="5" t="inlineStr"/>
-      <c r="Q131" s="5" t="inlineStr"/>
-      <c r="R131" s="6" t="inlineStr"/>
+      <c r="P131" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q131" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R131" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Haiku 5.5 high, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK.</t>
+        </is>
+      </c>
       <c r="S131" s="4" t="inlineStr"/>
     </row>
     <row r="132" ht="110" customHeight="1">
@@ -10467,9 +12007,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P132" s="5" t="inlineStr"/>
-      <c r="Q132" s="5" t="inlineStr"/>
-      <c r="R132" s="6" t="inlineStr"/>
+      <c r="P132" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q132" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R132" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S132" s="4" t="inlineStr"/>
     </row>
     <row r="133" ht="110" customHeight="1">
@@ -10544,9 +12096,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P133" s="5" t="inlineStr"/>
-      <c r="Q133" s="5" t="inlineStr"/>
-      <c r="R133" s="6" t="inlineStr"/>
+      <c r="P133" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q133" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R133" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S133" s="4" t="inlineStr"/>
     </row>
     <row r="134" ht="110" customHeight="1">
@@ -10621,9 +12185,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P134" s="5" t="inlineStr"/>
-      <c r="Q134" s="5" t="inlineStr"/>
-      <c r="R134" s="6" t="inlineStr"/>
+      <c r="P134" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q134" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R134" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S134" s="4" t="inlineStr"/>
     </row>
     <row r="135" ht="110" customHeight="1">
@@ -10698,9 +12274,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P135" s="5" t="inlineStr"/>
-      <c r="Q135" s="5" t="inlineStr"/>
-      <c r="R135" s="6" t="inlineStr"/>
+      <c r="P135" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q135" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R135" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S135" s="4" t="inlineStr"/>
     </row>
     <row r="136" ht="110" customHeight="1">
@@ -10775,9 +12363,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P136" s="5" t="inlineStr"/>
-      <c r="Q136" s="5" t="inlineStr"/>
-      <c r="R136" s="6" t="inlineStr"/>
+      <c r="P136" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q136" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R136" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: STATISTIK. Dinilai C1 dari definisi protokol; aturan Fatma untuk jenis ini belum ada, dan bila tidak dianggap C1 usul kode C2.</t>
+        </is>
+      </c>
       <c r="S136" s="4" t="inlineStr"/>
     </row>
     <row r="137" ht="110" customHeight="1">
@@ -10852,9 +12452,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P137" s="5" t="inlineStr"/>
-      <c r="Q137" s="5" t="inlineStr"/>
-      <c r="R137" s="6" t="inlineStr"/>
+      <c r="P137" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q137" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R137" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S137" s="4" t="inlineStr"/>
     </row>
     <row r="138" ht="110" customHeight="1">
@@ -10929,9 +12541,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P138" s="5" t="inlineStr"/>
-      <c r="Q138" s="5" t="inlineStr"/>
-      <c r="R138" s="6" t="inlineStr"/>
+      <c r="P138" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q138" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R138" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Haiku 5.5 high, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK.</t>
+        </is>
+      </c>
       <c r="S138" s="4" t="inlineStr"/>
     </row>
     <row r="139" ht="110" customHeight="1">
@@ -11006,9 +12630,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P139" s="5" t="inlineStr"/>
-      <c r="Q139" s="5" t="inlineStr"/>
-      <c r="R139" s="6" t="inlineStr"/>
+      <c r="P139" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q139" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R139" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Haiku 5.5 high, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme DATA (model M4+M3); akuisisi D (model V).</t>
+        </is>
+      </c>
       <c r="S139" s="4" t="inlineStr"/>
     </row>
     <row r="140" ht="110" customHeight="1">
@@ -11083,9 +12719,17 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P140" s="5" t="inlineStr"/>
+      <c r="P140" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="Q140" s="5" t="inlineStr"/>
-      <c r="R140" s="6" t="inlineStr"/>
+      <c r="R140" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: TIDAK_ADA. Bukan C1; usul kode C2.</t>
+        </is>
+      </c>
       <c r="S140" s="4" t="inlineStr"/>
     </row>
     <row r="141" ht="110" customHeight="1">
@@ -11160,9 +12804,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P141" s="5" t="inlineStr"/>
-      <c r="Q141" s="5" t="inlineStr"/>
-      <c r="R141" s="6" t="inlineStr"/>
+      <c r="P141" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q141" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R141" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Haiku 5.5 high, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK.</t>
+        </is>
+      </c>
       <c r="S141" s="4" t="inlineStr"/>
     </row>
     <row r="142" ht="110" customHeight="1">
@@ -11237,9 +12893,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P142" s="5" t="inlineStr"/>
-      <c r="Q142" s="5" t="inlineStr"/>
-      <c r="R142" s="6" t="inlineStr"/>
+      <c r="P142" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q142" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R142" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Haiku 5.5 high, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK.</t>
+        </is>
+      </c>
       <c r="S142" s="4" t="inlineStr"/>
     </row>
     <row r="143" ht="110" customHeight="1">
@@ -11314,9 +12982,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P143" s="5" t="inlineStr"/>
-      <c r="Q143" s="5" t="inlineStr"/>
-      <c r="R143" s="6" t="inlineStr"/>
+      <c r="P143" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q143" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R143" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: REKONSTRUKSI. Dinilai C1 dari definisi protokol; aturan Fatma untuk jenis ini belum ada, dan bila tidak dianggap C1 usul kode C5.</t>
+        </is>
+      </c>
       <c r="S143" s="4" t="inlineStr"/>
     </row>
     <row r="144" ht="110" customHeight="1">
@@ -11391,9 +13071,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P144" s="5" t="inlineStr"/>
-      <c r="Q144" s="5" t="inlineStr"/>
-      <c r="R144" s="6" t="inlineStr"/>
+      <c r="P144" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q144" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R144" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S144" s="4" t="inlineStr"/>
     </row>
     <row r="145" ht="110" customHeight="1">
@@ -11468,9 +13160,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P145" s="5" t="inlineStr"/>
-      <c r="Q145" s="5" t="inlineStr"/>
-      <c r="R145" s="6" t="inlineStr"/>
+      <c r="P145" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q145" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R145" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S145" s="4" t="inlineStr"/>
     </row>
     <row r="146" ht="110" customHeight="1">
@@ -11545,9 +13249,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P146" s="5" t="inlineStr"/>
-      <c r="Q146" s="5" t="inlineStr"/>
-      <c r="R146" s="6" t="inlineStr"/>
+      <c r="P146" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q146" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R146" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Haiku 5.5 high, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M3 (model M2+M3); per_kelas Y (model N).</t>
+        </is>
+      </c>
       <c r="S146" s="4" t="inlineStr"/>
     </row>
     <row r="147" ht="110" customHeight="1">
@@ -11622,9 +13338,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P147" s="5" t="inlineStr"/>
-      <c r="Q147" s="5" t="inlineStr"/>
-      <c r="R147" s="6" t="inlineStr"/>
+      <c r="P147" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q147" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R147" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S147" s="4" t="inlineStr"/>
     </row>
     <row r="148" ht="110" customHeight="1">
@@ -11699,9 +13427,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P148" s="5" t="inlineStr"/>
-      <c r="Q148" s="5" t="inlineStr"/>
-      <c r="R148" s="6" t="inlineStr"/>
+      <c r="P148" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q148" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R148" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S148" s="4" t="inlineStr"/>
     </row>
     <row r="149" ht="110" customHeight="1">
@@ -11776,9 +13516,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P149" s="5" t="inlineStr"/>
-      <c r="Q149" s="5" t="inlineStr"/>
-      <c r="R149" s="6" t="inlineStr"/>
+      <c r="P149" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q149" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R149" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S149" s="4" t="inlineStr"/>
     </row>
     <row r="150" ht="110" customHeight="1">
@@ -11853,9 +13605,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P150" s="5" t="inlineStr"/>
-      <c r="Q150" s="5" t="inlineStr"/>
-      <c r="R150" s="6" t="inlineStr"/>
+      <c r="P150" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q150" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R150" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S150" s="4" t="inlineStr"/>
     </row>
     <row r="151" ht="110" customHeight="1">
@@ -11930,9 +13694,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P151" s="5" t="inlineStr"/>
-      <c r="Q151" s="5" t="inlineStr"/>
-      <c r="R151" s="6" t="inlineStr"/>
+      <c r="P151" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q151" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R151" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S151" s="4" t="inlineStr"/>
     </row>
     <row r="152" ht="110" customHeight="1">
@@ -12007,9 +13783,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P152" s="5" t="inlineStr"/>
-      <c r="Q152" s="5" t="inlineStr"/>
-      <c r="R152" s="6" t="inlineStr"/>
+      <c r="P152" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q152" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R152" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: STATISTIK. Dinilai C1 dari definisi protokol; aturan Fatma untuk jenis ini belum ada, dan bila tidak dianggap C1 usul kode C4.</t>
+        </is>
+      </c>
       <c r="S152" s="4" t="inlineStr"/>
     </row>
     <row r="153" ht="110" customHeight="1">
@@ -12084,9 +13872,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P153" s="5" t="inlineStr"/>
-      <c r="Q153" s="5" t="inlineStr"/>
-      <c r="R153" s="6" t="inlineStr"/>
+      <c r="P153" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q153" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R153" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S153" s="4" t="inlineStr"/>
     </row>
     <row r="154" ht="110" customHeight="1">
@@ -12161,9 +13961,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P154" s="5" t="inlineStr"/>
-      <c r="Q154" s="5" t="inlineStr"/>
-      <c r="R154" s="6" t="inlineStr"/>
+      <c r="P154" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q154" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R154" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S154" s="4" t="inlineStr"/>
     </row>
     <row r="155" ht="110" customHeight="1">
@@ -12238,9 +14050,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P155" s="5" t="inlineStr"/>
-      <c r="Q155" s="5" t="inlineStr"/>
-      <c r="R155" s="6" t="inlineStr"/>
+      <c r="P155" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q155" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R155" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S155" s="4" t="inlineStr"/>
     </row>
     <row r="156" ht="110" customHeight="1">
@@ -12315,9 +14139,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P156" s="5" t="inlineStr"/>
-      <c r="Q156" s="5" t="inlineStr"/>
-      <c r="R156" s="6" t="inlineStr"/>
+      <c r="P156" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q156" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R156" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S156" s="4" t="inlineStr"/>
     </row>
     <row r="157" ht="110" customHeight="1">
@@ -12392,9 +14228,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P157" s="5" t="inlineStr"/>
-      <c r="Q157" s="5" t="inlineStr"/>
-      <c r="R157" s="6" t="inlineStr"/>
+      <c r="P157" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q157" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R157" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S157" s="4" t="inlineStr"/>
     </row>
     <row r="158" ht="110" customHeight="1">
@@ -12469,9 +14317,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P158" s="5" t="inlineStr"/>
-      <c r="Q158" s="5" t="inlineStr"/>
-      <c r="R158" s="6" t="inlineStr"/>
+      <c r="P158" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q158" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R158" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S158" s="4" t="inlineStr"/>
     </row>
     <row r="159" ht="110" customHeight="1">
@@ -12546,9 +14406,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P159" s="5" t="inlineStr"/>
-      <c r="Q159" s="5" t="inlineStr"/>
-      <c r="R159" s="6" t="inlineStr"/>
+      <c r="P159" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q159" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R159" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: REKONSTRUKSI. Dinilai C1 dari definisi protokol; aturan Fatma untuk jenis ini belum ada, dan bila tidak dianggap C1 usul kode C5. Usul koreksi kode: akuisisi S menjadi D.</t>
+        </is>
+      </c>
       <c r="S159" s="4" t="inlineStr"/>
     </row>
     <row r="160" ht="110" customHeight="1">
@@ -12623,9 +14495,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P160" s="5" t="inlineStr"/>
-      <c r="Q160" s="5" t="inlineStr"/>
-      <c r="R160" s="6" t="inlineStr"/>
+      <c r="P160" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q160" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R160" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S160" s="4" t="inlineStr"/>
     </row>
     <row r="161" ht="110" customHeight="1">
@@ -12700,9 +14584,17 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P161" s="5" t="inlineStr"/>
+      <c r="P161" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="Q161" s="5" t="inlineStr"/>
-      <c r="R161" s="6" t="inlineStr"/>
+      <c r="R161" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Haiku 5.5 high, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: TIDAK_ADA. Bukan C1; usul kode C5.</t>
+        </is>
+      </c>
       <c r="S161" s="4" t="inlineStr"/>
     </row>
     <row r="162" ht="110" customHeight="1">
@@ -12777,9 +14669,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P162" s="5" t="inlineStr"/>
-      <c r="Q162" s="5" t="inlineStr"/>
-      <c r="R162" s="6" t="inlineStr"/>
+      <c r="P162" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q162" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R162" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: REKONSTRUKSI. Dinilai C1 dari definisi protokol; aturan Fatma untuk jenis ini belum ada, dan bila tidak dianggap C1 usul kode C5. Usul koreksi kode: akuisisi S menjadi D.</t>
+        </is>
+      </c>
       <c r="S162" s="4" t="inlineStr"/>
     </row>
     <row r="163" ht="110" customHeight="1">
@@ -12854,9 +14758,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P163" s="5" t="inlineStr"/>
-      <c r="Q163" s="5" t="inlineStr"/>
-      <c r="R163" s="6" t="inlineStr"/>
+      <c r="P163" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q163" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R163" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: REKONSTRUKSI. Dinilai C1 dari definisi protokol; aturan Fatma untuk jenis ini belum ada, dan bila tidak dianggap C1 usul kode C2. Usul koreksi kode: akuisisi V menjadi D.</t>
+        </is>
+      </c>
       <c r="S163" s="4" t="inlineStr"/>
     </row>
     <row r="164" ht="110" customHeight="1">
@@ -12931,9 +14847,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P164" s="5" t="inlineStr"/>
-      <c r="Q164" s="5" t="inlineStr"/>
-      <c r="R164" s="6" t="inlineStr"/>
+      <c r="P164" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q164" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R164" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK.</t>
+        </is>
+      </c>
       <c r="S164" s="4" t="inlineStr"/>
     </row>
     <row r="165" ht="110" customHeight="1">
@@ -13008,9 +14936,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P165" s="5" t="inlineStr"/>
-      <c r="Q165" s="5" t="inlineStr"/>
-      <c r="R165" s="6" t="inlineStr"/>
+      <c r="P165" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q165" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R165" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: REKONSTRUKSI. Dinilai C1 dari definisi protokol; aturan Fatma untuk jenis ini belum ada, dan bila tidak dianggap C1 usul kode C5. Kode sama dengan penilai; pemeriksa mengusulkan mekanisme M1+M4 (regresi kalibrasi dihitung sebagai M1).</t>
+        </is>
+      </c>
       <c r="S165" s="4" t="inlineStr"/>
     </row>
     <row r="166" ht="110" customHeight="1">
@@ -13085,9 +15025,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P166" s="5" t="inlineStr"/>
-      <c r="Q166" s="5" t="inlineStr"/>
-      <c r="R166" s="6" t="inlineStr"/>
+      <c r="P166" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q166" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R166" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK.</t>
+        </is>
+      </c>
       <c r="S166" s="4" t="inlineStr"/>
     </row>
     <row r="167" ht="110" customHeight="1">
@@ -13162,9 +15114,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P167" s="5" t="inlineStr"/>
-      <c r="Q167" s="5" t="inlineStr"/>
-      <c r="R167" s="6" t="inlineStr"/>
+      <c r="P167" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q167" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R167" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: REKONSTRUKSI. Dinilai C1 dari definisi protokol; aturan Fatma untuk jenis ini belum ada, dan bila tidak dianggap C1 usul kode C5.  Artikel data tanpa metode hitung; perlakuannya perlu seragam dengan no 168.</t>
+        </is>
+      </c>
       <c r="S167" s="4" t="inlineStr"/>
     </row>
     <row r="168" ht="110" customHeight="1">
@@ -13241,7 +15205,11 @@
       </c>
       <c r="P168" s="5" t="inlineStr"/>
       <c r="Q168" s="5" t="inlineStr"/>
-      <c r="R168" s="6" t="inlineStr"/>
+      <c r="R168" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5 (12 Oktober 2026) dan verifikasinya tidak sepakat: penilai N (usul kode C5), pemeriksa Y dengan keyakinan rendah. Artikel data tanpa metode hitung; perlu keputusan peninjau, seragam dengan no 167.</t>
+        </is>
+      </c>
       <c r="S168" s="4" t="inlineStr"/>
     </row>
     <row r="169" ht="110" customHeight="1">
@@ -13316,9 +15284,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P169" s="5" t="inlineStr"/>
-      <c r="Q169" s="5" t="inlineStr"/>
-      <c r="R169" s="6" t="inlineStr"/>
+      <c r="P169" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q169" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R169" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S169" s="4" t="inlineStr"/>
     </row>
     <row r="170" ht="110" customHeight="1">
@@ -13393,9 +15373,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P170" s="5" t="inlineStr"/>
-      <c r="Q170" s="5" t="inlineStr"/>
-      <c r="R170" s="6" t="inlineStr"/>
+      <c r="P170" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q170" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R170" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S170" s="4" t="inlineStr"/>
     </row>
     <row r="171" ht="110" customHeight="1">
@@ -13470,9 +15462,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P171" s="5" t="inlineStr"/>
-      <c r="Q171" s="5" t="inlineStr"/>
-      <c r="R171" s="6" t="inlineStr"/>
+      <c r="P171" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q171" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R171" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S171" s="4" t="inlineStr"/>
     </row>
     <row r="172" ht="110" customHeight="1">
@@ -13547,9 +15551,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P172" s="5" t="inlineStr"/>
-      <c r="Q172" s="5" t="inlineStr"/>
-      <c r="R172" s="6" t="inlineStr"/>
+      <c r="P172" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q172" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R172" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Haiku 5.5 high, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M3+M4 (model M2+M3).</t>
+        </is>
+      </c>
       <c r="S172" s="4" t="inlineStr"/>
     </row>
     <row r="173" ht="110" customHeight="1">
@@ -13624,9 +15640,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P173" s="5" t="inlineStr"/>
-      <c r="Q173" s="5" t="inlineStr"/>
-      <c r="R173" s="6" t="inlineStr"/>
+      <c r="P173" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q173" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R173" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S173" s="4" t="inlineStr"/>
     </row>
     <row r="174" ht="110" customHeight="1">
@@ -13701,9 +15729,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P174" s="5" t="inlineStr"/>
-      <c r="Q174" s="5" t="inlineStr"/>
-      <c r="R174" s="6" t="inlineStr"/>
+      <c r="P174" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q174" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R174" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S174" s="4" t="inlineStr"/>
     </row>
     <row r="175" ht="110" customHeight="1">
@@ -13778,9 +15818,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P175" s="5" t="inlineStr"/>
-      <c r="Q175" s="5" t="inlineStr"/>
-      <c r="R175" s="6" t="inlineStr"/>
+      <c r="P175" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q175" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R175" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S175" s="4" t="inlineStr"/>
     </row>
     <row r="176" ht="110" customHeight="1">
@@ -13855,9 +15907,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P176" s="5" t="inlineStr"/>
-      <c r="Q176" s="5" t="inlineStr"/>
-      <c r="R176" s="6" t="inlineStr"/>
+      <c r="P176" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q176" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R176" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S176" s="4" t="inlineStr"/>
     </row>
     <row r="177" ht="110" customHeight="1">
@@ -13932,9 +15996,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P177" s="5" t="inlineStr"/>
-      <c r="Q177" s="5" t="inlineStr"/>
-      <c r="R177" s="6" t="inlineStr"/>
+      <c r="P177" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q177" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R177" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S177" s="4" t="inlineStr"/>
     </row>
     <row r="178" ht="110" customHeight="1">
@@ -14009,9 +16085,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P178" s="5" t="inlineStr"/>
-      <c r="Q178" s="5" t="inlineStr"/>
-      <c r="R178" s="6" t="inlineStr"/>
+      <c r="P178" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q178" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R178" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S178" s="4" t="inlineStr"/>
     </row>
     <row r="179" ht="110" customHeight="1">
@@ -14086,9 +16174,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P179" s="5" t="inlineStr"/>
-      <c r="Q179" s="5" t="inlineStr"/>
-      <c r="R179" s="6" t="inlineStr"/>
+      <c r="P179" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q179" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R179" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S179" s="4" t="inlineStr"/>
     </row>
     <row r="180" ht="110" customHeight="1">
@@ -14163,9 +16263,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P180" s="5" t="inlineStr"/>
-      <c r="Q180" s="5" t="inlineStr"/>
-      <c r="R180" s="6" t="inlineStr"/>
+      <c r="P180" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q180" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R180" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Haiku 5.5 high, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: akuisisi V (model D).</t>
+        </is>
+      </c>
       <c r="S180" s="4" t="inlineStr"/>
     </row>
     <row r="181" ht="110" customHeight="1">
@@ -14240,9 +16352,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P181" s="5" t="inlineStr"/>
-      <c r="Q181" s="5" t="inlineStr"/>
-      <c r="R181" s="6" t="inlineStr"/>
+      <c r="P181" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q181" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R181" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S181" s="4" t="inlineStr"/>
     </row>
     <row r="182" ht="110" customHeight="1">
@@ -14317,9 +16441,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P182" s="5" t="inlineStr"/>
-      <c r="Q182" s="5" t="inlineStr"/>
-      <c r="R182" s="6" t="inlineStr"/>
+      <c r="P182" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q182" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R182" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S182" s="4" t="inlineStr"/>
     </row>
     <row r="183" ht="110" customHeight="1">
@@ -14394,9 +16530,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P183" s="5" t="inlineStr"/>
-      <c r="Q183" s="5" t="inlineStr"/>
-      <c r="R183" s="6" t="inlineStr"/>
+      <c r="P183" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q183" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R183" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul koreksi kode: mekanisme M1 menjadi M1+M4.</t>
+        </is>
+      </c>
       <c r="S183" s="4" t="inlineStr"/>
     </row>
     <row r="184" ht="110" customHeight="1">
@@ -14471,9 +16619,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P184" s="5" t="inlineStr"/>
-      <c r="Q184" s="5" t="inlineStr"/>
-      <c r="R184" s="6" t="inlineStr"/>
+      <c r="P184" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q184" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R184" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S184" s="4" t="inlineStr"/>
     </row>
     <row r="185" ht="110" customHeight="1">
@@ -14548,9 +16708,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P185" s="5" t="inlineStr"/>
-      <c r="Q185" s="5" t="inlineStr"/>
-      <c r="R185" s="6" t="inlineStr"/>
+      <c r="P185" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q185" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R185" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Haiku 5.5 high, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M2 (model M1); akuisisi T (model D).</t>
+        </is>
+      </c>
       <c r="S185" s="4" t="inlineStr"/>
     </row>
     <row r="186" ht="110" customHeight="1">
@@ -14625,9 +16797,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P186" s="5" t="inlineStr"/>
-      <c r="Q186" s="5" t="inlineStr"/>
-      <c r="R186" s="6" t="inlineStr"/>
+      <c r="P186" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q186" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R186" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S186" s="4" t="inlineStr"/>
     </row>
     <row r="187" ht="110" customHeight="1">
@@ -14698,9 +16882,21 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P187" s="5" t="inlineStr"/>
-      <c r="Q187" s="5" t="inlineStr"/>
-      <c r="R187" s="6" t="inlineStr"/>
+      <c r="P187" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q187" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R187" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S187" s="4" t="inlineStr"/>
     </row>
     <row r="188" ht="110" customHeight="1">
@@ -14775,9 +16971,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P188" s="5" t="inlineStr"/>
-      <c r="Q188" s="5" t="inlineStr"/>
-      <c r="R188" s="6" t="inlineStr"/>
+      <c r="P188" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q188" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R188" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S188" s="4" t="inlineStr"/>
     </row>
     <row r="189" ht="110" customHeight="1">
@@ -14852,9 +17060,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P189" s="5" t="inlineStr"/>
-      <c r="Q189" s="5" t="inlineStr"/>
-      <c r="R189" s="6" t="inlineStr"/>
+      <c r="P189" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q189" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R189" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S189" s="4" t="inlineStr"/>
     </row>
     <row r="190" ht="110" customHeight="1">
@@ -14929,9 +17149,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P190" s="5" t="inlineStr"/>
-      <c r="Q190" s="5" t="inlineStr"/>
-      <c r="R190" s="6" t="inlineStr"/>
+      <c r="P190" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q190" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R190" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S190" s="4" t="inlineStr"/>
     </row>
     <row r="191" ht="110" customHeight="1">
@@ -15002,9 +17234,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P191" s="5" t="inlineStr"/>
-      <c r="Q191" s="5" t="inlineStr"/>
-      <c r="R191" s="6" t="inlineStr"/>
+      <c r="P191" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q191" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R191" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S191" s="4" t="inlineStr"/>
     </row>
     <row r="192" ht="110" customHeight="1">
@@ -15079,9 +17323,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P192" s="5" t="inlineStr"/>
-      <c r="Q192" s="5" t="inlineStr"/>
-      <c r="R192" s="6" t="inlineStr"/>
+      <c r="P192" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q192" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R192" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S192" s="4" t="inlineStr"/>
     </row>
     <row r="193" ht="110" customHeight="1">
@@ -15152,9 +17408,17 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P193" s="5" t="inlineStr"/>
+      <c r="P193" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="Q193" s="5" t="inlineStr"/>
-      <c r="R193" s="6" t="inlineStr"/>
+      <c r="R193" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: TIDAK_ADA. Bukan C1; usul kode C2.</t>
+        </is>
+      </c>
       <c r="S193" s="4" t="inlineStr"/>
     </row>
     <row r="194" ht="110" customHeight="1">
@@ -15225,9 +17489,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P194" s="5" t="inlineStr"/>
-      <c r="Q194" s="5" t="inlineStr"/>
-      <c r="R194" s="6" t="inlineStr"/>
+      <c r="P194" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q194" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R194" s="6" t="inlineStr">
+        <is>
+          <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: REKONSTRUKSI. Dinilai C1 dari definisi protokol; aturan Fatma untuk jenis ini belum ada, dan bila tidak dianggap C1 usul kode C5.</t>
+        </is>
+      </c>
       <c r="S194" s="4" t="inlineStr"/>
     </row>
     <row r="195" ht="110" customHeight="1">
@@ -15302,9 +17578,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P195" s="5" t="inlineStr"/>
-      <c r="Q195" s="5" t="inlineStr"/>
-      <c r="R195" s="6" t="inlineStr"/>
+      <c r="P195" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q195" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R195" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S195" s="4" t="inlineStr"/>
     </row>
     <row r="196" ht="110" customHeight="1">
@@ -15379,9 +17667,21 @@
           <t>N</t>
         </is>
       </c>
-      <c r="P196" s="5" t="inlineStr"/>
-      <c r="Q196" s="5" t="inlineStr"/>
-      <c r="R196" s="6" t="inlineStr"/>
+      <c r="P196" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q196" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R196" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
+        </is>
+      </c>
       <c r="S196" s="4" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cek 1: putuskan 118 perbedaan sampel buta; laporkan Cek 1 di naskah
- Ajudikasi 118 perbedaan nonkritis: dua pembaca buta Haiku 5.5 + penengah,
  diperiksa agen utama atas penyerahan peninjau. Delapan keputusan berubah
  (abstrak_V00.txt, log_perubahan.csv); korpus 1.000 kajian
  (C2 237, C4 50, C5 134).
- Bangun ulang matriks bukti, gambar, lampiran, makro angka, bib, katalog PDF;
  kompilasi main6.pdf.
- Naskah: paragraf sampel buta penulis pertama (kappa 0,57 dan 0,45) dan
  keterbatasan ketiga, dengan makro baru dari angka_naskah.py.
- Lembar Cek 2, Cek 5, dan Cek 6 disegarkan; id klaim draf Cek 6 dipetakan
  ulang; TUGAS, README, SERAH-TERIMA, PROTOKOL, dan AGENTS §3 diperbarui.
</commit_message>
<xml_diff>
--- a/literature/scopus-2026-09/verifikasi/cek-2-cek-tangan/cek_C1.xlsx
+++ b/literature/scopus-2026-09/verifikasi/cek-2-cek-tangan/cek_C1.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="keterangan" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'cek'!$A$1:$S$196</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'cek'!$A$1:$S$198</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S196"/>
+  <dimension ref="A1:S198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3514,7 +3514,11 @@
           <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: TIDAK_ADA. Bukan C1; usul kode X.</t>
         </is>
       </c>
-      <c r="S36" s="4" t="inlineStr"/>
+      <c r="S36" s="4" t="inlineStr">
+        <is>
+          <t>tidak lagi C1 di sumber (kini X E1); baris dipertahankan karena sudah diisi peninjau</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="110" customHeight="1">
       <c r="A37" s="3" t="n">
@@ -14595,7 +14599,11 @@
           <t>Penilaian buta Haiku 5.5 high, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: TIDAK_ADA. Bukan C1; usul kode C5.</t>
         </is>
       </c>
-      <c r="S161" s="4" t="inlineStr"/>
+      <c r="S161" s="4" t="inlineStr">
+        <is>
+          <t>tidak lagi C1 di sumber (kini C5); baris dipertahankan karena sudah diisi peninjau</t>
+        </is>
+      </c>
     </row>
     <row r="162" ht="110" customHeight="1">
       <c r="A162" s="3" t="n">
@@ -17684,13 +17692,183 @@
       </c>
       <c r="S196" s="4" t="inlineStr"/>
     </row>
+    <row r="197" ht="110" customHeight="1">
+      <c r="A197" s="3" t="n">
+        <v>198</v>
+      </c>
+      <c r="B197" s="3" t="n">
+        <v>131</v>
+      </c>
+      <c r="C197" s="3" t="inlineStr">
+        <is>
+          <t>timprae2025tomato</t>
+        </is>
+      </c>
+      <c r="D197" s="3" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E197" s="4" t="inlineStr">
+        <is>
+          <t>Tomato Growth Monitoring and Phenological Analysis Using Deep Learning-Based Instance Segmentation and 3D Point Cloud Reconstruction</t>
+        </is>
+      </c>
+      <c r="F197" s="3" t="inlineStr">
+        <is>
+          <t>10.3390/su172210120</t>
+        </is>
+      </c>
+      <c r="G197" s="4" t="inlineStr">
+        <is>
+          <t>Accurate and nondestructive monitoring of tomato growth is essential for large-scale greenhouse production; however, it remains challenging for small-fruited cultivars such as cherry tomatoes. Traditional 2D image analysis often fails to capture precise morphological traits, limiting its usefulness in growth modeling and yield estimation. This study proposes an automated phenotyping framework that integrates deep learning-based instance segmentation with high-resolution 3D point cloud reconstruction and ellipsoid fitting to estimate fruit size and ripeness from daily video recordings. These techniques enable accurate camera pose estimation and dense geometric reconstruction (via SfM and MVS), while Nerfacto enhances surface continuity and photorealistic fidelity, resulting in highly precise and visually consistent 3D representations. The reconstructed models are followed by CIELAB color analysis and logistic curve fitting to characterize the growth dynamics. When applied to real greenhouse conditions, the method achieved an average size estimation error of 8.01% compared to manual caliper measurements. During summer, the maximum growth rate (gmax) of size and ripeness were 24.14%, and 95.24% higher than in winter, respectively. Seasonal analysis revealed that winter-grown tomatoes matured approximately 10 days later than summer-grown fruits, highlighting environmental influences on phenological development. By enabling precise, noninvasive tracking of size and ripeness progression, this approach is a novel tool for smart and sustainable agriculture.</t>
+        </is>
+      </c>
+      <c r="H197" s="3" t="inlineStr">
+        <is>
+          <t>abstrak</t>
+        </is>
+      </c>
+      <c r="I197" s="3" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="J197" s="3" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="K197" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L197" s="4" t="inlineStr">
+        <is>
+          <t>tomat ceri rumah kaca; segmentasi instans + SfM/MVS + Nerfacto dari video harian; galat ukuran rata-rata 8,01% terhadap jangka sorong</t>
+        </is>
+      </c>
+      <c r="M197" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N197" s="3" t="inlineStr">
+        <is>
+          <t>literature/scopus-2026-09/teks/timprae2025tomato.txt</t>
+        </is>
+      </c>
+      <c r="O197" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P197" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q197" s="5" t="inlineStr"/>
+      <c r="R197" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 18 Oktober 2026 dari ajudikasi Cek 1 (dua pembaca buta Haiku 5.5 + penengah, diperiksa agen utama; diserahkan peninjau), cek-1-sampel-buta/ajudikasi/ajudikasi_cek1.csv. Isian model, bukan bacaan peninjau. Model 3D SfM/MVS dari video harian; aturan rekonstruksi 3D (TUGAS 1.1).</t>
+        </is>
+      </c>
+      <c r="S197" s="4" t="inlineStr"/>
+    </row>
+    <row r="198" ht="110" customHeight="1">
+      <c r="A198" s="3" t="n">
+        <v>199</v>
+      </c>
+      <c r="B198" s="3" t="n">
+        <v>570</v>
+      </c>
+      <c r="C198" s="3" t="inlineStr">
+        <is>
+          <t>seo2021development</t>
+        </is>
+      </c>
+      <c r="D198" s="3" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="E198" s="4" t="inlineStr">
+        <is>
+          <t>Development of monitoring robot system for tomato fruits in hydroponic greenhouses</t>
+        </is>
+      </c>
+      <c r="F198" s="3" t="inlineStr">
+        <is>
+          <t>10.3390/agronomy11112211</t>
+        </is>
+      </c>
+      <c r="G198" s="4" t="inlineStr">
+        <is>
+          <t>Crop monitoring is highly important in terms of the efficient and stable performance of tasks such as planting, spraying, and harvesting, and for this reason, several studies are being conducted to develop and improve crop monitoring robots. In addition, the applications of deep learning algorithms are increasing in the development of agricultural robots since deep learning algorithms that use convolutional neural networks have been proven to show outstanding performance in image classification, segmentation, and object detection. However, most of these applications are focused on the development of harvesting robots, and thus, there are only a few studies that improve and develop monitoring robots through the use of deep learning. For this reason, we aimed to develop a real-time robot monitoring system for the generative growth of tomatoes. The presented method detects tomato fruits grown in hydroponic greenhouses using the Faster R-CNN (region-based convolutional neural network). In addition, we sought to select a color model that was robust to external light, and we used hue values to develop an image-based maturity standard for tomato fruits; furthermore, the developed maturity standard was verified through comparison with expert classification. Finally, the number of tomatoes was counted using a centroid-based tracking algorithm. We trained the detection model using an open dataset and tested the whole system in real-time in a hydroponic greenhouse. A total of 53 tomato fruits were used to verify the developed system, and the developed system achieved 88.6% detection accuracy when completely obscured fruits not captured by the camera were included. When excluding obscured fruits, the system’s accuracy was 90.2%. For the maturity classification, we conducted qualitative evaluations with the assistance of experts.</t>
+        </is>
+      </c>
+      <c r="H198" s="3" t="inlineStr">
+        <is>
+          <t>abstrak</t>
+        </is>
+      </c>
+      <c r="I198" s="3" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="J198" s="3" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="K198" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L198" s="4" t="inlineStr">
+        <is>
+          <t>tomat hidroponik, robot; Faster R-CNN + standar kematangan hue; hitung dengan pelacakan centroid; akurasi deteksi 88,6% (53 buah)</t>
+        </is>
+      </c>
+      <c r="M198" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N198" s="3" t="inlineStr">
+        <is>
+          <t>literature/scopus-2026-09/teks/seo2021development.txt</t>
+        </is>
+      </c>
+      <c r="O198" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P198" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q198" s="5" t="inlineStr"/>
+      <c r="R198" s="6" t="inlineStr">
+        <is>
+          <t>Diisi 18 Oktober 2026 dari ajudikasi Cek 1 (dua pembaca buta Haiku 5.5 + penengah, diperiksa agen utama; diserahkan peninjau), cek-1-sampel-buta/ajudikasi/ajudikasi_cek1.csv. Isian model, bukan bacaan peninjau. Hitungan dengan pelacakan centroid antar-frame.</t>
+        </is>
+      </c>
+      <c r="S198" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S196"/>
+  <autoFilter ref="A1:S198"/>
   <dataValidations count="2">
-    <dataValidation sqref="P2:P396" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak sah" error="Pilih salah satu: Y,N" type="list">
+    <dataValidation sqref="P2:P398" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak sah" error="Pilih salah satu: Y,N" type="list">
       <formula1>"Y,N"</formula1>
     </dataValidation>
-    <dataValidation sqref="Q2:Q396" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak sah" error="Pilih salah satu: Y,N" type="list">
+    <dataValidation sqref="Q2:Q398" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak sah" error="Pilih salah satu: Y,N" type="list">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Verifikasi main6: putuskan butir TUGAS, kode ulang buta C1/C3, cek fakta naskah
- Aturan pengodean baru (rekonstruksi 3D, gabungan statistik, pelacakan tanpa
  evaluasi, kalibrasi, akuisisi S/T, set data, E7, lokasi C3) di PROTOKOL.md
  dan bagian metode naskah.
- 87 rekaman dibaca ulang buta; 26 keputusan di abstrak_W00.txt. Korpus:
  1.013 kajian Scopus + 5 dari luar pencarian (L2-L5 dari daftar pustaka).
- Semua kajian C1 dan C3 dikode ulang buta; label C1 diterapkan lewat Cek 5,
  label C3 ke kode_C3.txt.
- Cek fakta seluruh baris kosong: 190 pasangan diperiksa buta, 65 klaim
  diperbaiki di naskah; lembar cek_fakta.csv terisi penuh.
- Bangun ulang angka, gambar, lampiran, daftar pustaka; kompilasi main6.pdf
  (34 halaman).
- TUGAS.md kini hanya memuat F.4 dan 5.7; draf lama dipindah ke
  putaran-kedua/draf-cek/.
</commit_message>
<xml_diff>
--- a/literature/scopus-2026-09/verifikasi/cek-2-cek-tangan/cek_C1.xlsx
+++ b/literature/scopus-2026-09/verifikasi/cek-2-cek-tangan/cek_C1.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="keterangan" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'cek'!$A$1:$S$198</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'cek'!$A$1:$S$204</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S198"/>
+  <dimension ref="A1:S204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -652,7 +652,11 @@
           <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
         </is>
       </c>
-      <c r="S2" s="4" t="inlineStr"/>
+      <c r="S2" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M2+M3'</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="110" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -907,7 +911,11 @@
           <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
         </is>
       </c>
-      <c r="S5" s="4" t="inlineStr"/>
+      <c r="S5" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M2+M3'</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="110" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -1413,7 +1421,11 @@
           <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M4 (model M3).</t>
         </is>
       </c>
-      <c r="S11" s="4" t="inlineStr"/>
+      <c r="S11" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M4'; akuisisi_ai='S'</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="110" customHeight="1">
       <c r="A12" s="3" t="n">
@@ -1668,7 +1680,11 @@
           <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
         </is>
       </c>
-      <c r="S14" s="4" t="inlineStr"/>
+      <c r="S14" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M2+M3'</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="110" customHeight="1">
       <c r="A15" s="3" t="n">
@@ -1753,7 +1769,11 @@
           <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M2+M3 (model M3); per_kelas Y (model N).</t>
         </is>
       </c>
-      <c r="S15" s="4" t="inlineStr"/>
+      <c r="S15" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M2+M3'; per_kelas_ai='Y'</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="110" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -1923,7 +1943,11 @@
           <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
         </is>
       </c>
-      <c r="S17" s="4" t="inlineStr"/>
+      <c r="S17" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M2+M3'</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="110" customHeight="1">
       <c r="A18" s="3" t="n">
@@ -2166,7 +2190,11 @@
           <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: STATISTIK. Dinilai C1 dari definisi protokol; aturan Fatma untuk jenis ini belum ada, dan bila tidak dianggap C1 usul kode C2. Usul koreksi kode: mekanisme M4 menjadi M1; per_kelas Y menjadi N.</t>
         </is>
       </c>
-      <c r="S20" s="4" t="inlineStr"/>
+      <c r="S20" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M1'</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="110" customHeight="1">
       <c r="A21" s="3" t="n">
@@ -2336,7 +2364,11 @@
           <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M4 (model M0).</t>
         </is>
       </c>
-      <c r="S22" s="4" t="inlineStr"/>
+      <c r="S22" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M4'; akuisisi_ai='V'</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="110" customHeight="1">
       <c r="A23" s="3" t="n">
@@ -2417,7 +2449,11 @@
           <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK.</t>
         </is>
       </c>
-      <c r="S23" s="4" t="inlineStr"/>
+      <c r="S23" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: per_kelas_ai='Y'</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="110" customHeight="1">
       <c r="A24" s="3" t="n">
@@ -2502,7 +2538,11 @@
           <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
         </is>
       </c>
-      <c r="S24" s="4" t="inlineStr"/>
+      <c r="S24" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M3+M4'; akuisisi_ai='S'</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="110" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -2672,7 +2712,11 @@
           <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M2+M3 (model M3).</t>
         </is>
       </c>
-      <c r="S26" s="4" t="inlineStr"/>
+      <c r="S26" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M2+M3'</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="110" customHeight="1">
       <c r="A27" s="3" t="n">
@@ -3348,7 +3392,11 @@
           <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M2+M3 (model M3).</t>
         </is>
       </c>
-      <c r="S34" s="4" t="inlineStr"/>
+      <c r="S34" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M2+M3'</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="110" customHeight="1">
       <c r="A35" s="3" t="n">
@@ -3433,7 +3481,11 @@
           <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: REKONSTRUKSI. Dinilai C1 dari definisi protokol; aturan Fatma untuk jenis ini belum ada, dan bila tidak dianggap C1 usul kode C2. Usul koreksi kode: mekanisme M0 menjadi M4.</t>
         </is>
       </c>
-      <c r="S35" s="4" t="inlineStr"/>
+      <c r="S35" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M4'</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="110" customHeight="1">
       <c r="A36" s="3" t="n">
@@ -3599,7 +3651,11 @@
           <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: REKONSTRUKSI. Dinilai C1 dari definisi protokol; aturan Fatma untuk jenis ini belum ada, dan bila tidak dianggap C1 usul kode C5.</t>
         </is>
       </c>
-      <c r="S37" s="4" t="inlineStr"/>
+      <c r="S37" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: akuisisi_ai='S'</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="110" customHeight="1">
       <c r="A38" s="3" t="n">
@@ -3769,7 +3825,11 @@
           <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: per_kelas Y (model N).</t>
         </is>
       </c>
-      <c r="S39" s="4" t="inlineStr"/>
+      <c r="S39" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: per_kelas_ai='Y'</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="110" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -3854,7 +3914,11 @@
           <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: STATISTIK. Dinilai C1 dari definisi protokol; aturan Fatma untuk jenis ini belum ada, dan bila tidak dianggap C1 usul kode C2. Usul koreksi kode: mekanisme M1+M4 menjadi M1.</t>
         </is>
       </c>
-      <c r="S40" s="4" t="inlineStr"/>
+      <c r="S40" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M1'</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="110" customHeight="1">
       <c r="A41" s="3" t="n">
@@ -4194,7 +4258,11 @@
           <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
         </is>
       </c>
-      <c r="S44" s="4" t="inlineStr"/>
+      <c r="S44" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: akuisisi_ai='S'</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="110" customHeight="1">
       <c r="A45" s="3" t="n">
@@ -4372,7 +4440,11 @@
           <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M1+M3 (model M3+M4).</t>
         </is>
       </c>
-      <c r="S46" s="4" t="inlineStr"/>
+      <c r="S46" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M3'</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="110" customHeight="1">
       <c r="A47" s="3" t="n">
@@ -4730,7 +4802,11 @@
           <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
         </is>
       </c>
-      <c r="S50" s="4" t="inlineStr"/>
+      <c r="S50" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: akuisisi_ai='S'</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="110" customHeight="1">
       <c r="A51" s="3" t="n">
@@ -4908,7 +4984,11 @@
           <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: REKONSTRUKSI. Dinilai C1 dari definisi protokol; aturan Fatma untuk jenis ini belum ada, dan bila tidak dianggap C1 usul kode C5. Usul koreksi kode: mekanisme M4+M1 menjadi M4; akuisisi S menjadi D.</t>
         </is>
       </c>
-      <c r="S52" s="4" t="inlineStr"/>
+      <c r="S52" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M4'</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="110" customHeight="1">
       <c r="A53" s="3" t="n">
@@ -4997,7 +5077,11 @@
           <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M2+M3 (model M3+M4).</t>
         </is>
       </c>
-      <c r="S53" s="4" t="inlineStr"/>
+      <c r="S53" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M2+M3'</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="110" customHeight="1">
       <c r="A54" s="3" t="n">
@@ -5442,7 +5526,11 @@
           <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
         </is>
       </c>
-      <c r="S58" s="4" t="inlineStr"/>
+      <c r="S58" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: akuisisi_ai='S'</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="110" customHeight="1">
       <c r="A59" s="3" t="n">
@@ -5620,7 +5708,11 @@
           <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M2+M3 (model M3); per_kelas Y (model N).</t>
         </is>
       </c>
-      <c r="S60" s="4" t="inlineStr"/>
+      <c r="S60" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M2+M3'; per_kelas_ai='Y'</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="110" customHeight="1">
       <c r="A61" s="3" t="n">
@@ -5889,7 +5981,11 @@
           <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: REKONSTRUKSI. Dinilai C1 dari definisi protokol; aturan Fatma untuk jenis ini belum ada, dan bila tidak dianggap C1 usul kode C5. Usul koreksi kode: mekanisme M4+M5 menjadi M4.</t>
         </is>
       </c>
-      <c r="S63" s="4" t="inlineStr"/>
+      <c r="S63" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: akuisisi_ai='S'</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="110" customHeight="1">
       <c r="A64" s="3" t="n">
@@ -5978,7 +6074,11 @@
           <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: REKONSTRUKSI. Dinilai C1 dari definisi protokol; aturan Fatma untuk jenis ini belum ada, dan bila tidak dianggap C1 usul kode C5.</t>
         </is>
       </c>
-      <c r="S64" s="4" t="inlineStr"/>
+      <c r="S64" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: akuisisi_ai='S'</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="110" customHeight="1">
       <c r="A65" s="3" t="n">
@@ -6156,7 +6256,11 @@
           <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: per_kelas N (model Y).</t>
         </is>
       </c>
-      <c r="S66" s="4" t="inlineStr"/>
+      <c r="S66" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: per_kelas_ai='N'</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="110" customHeight="1">
       <c r="A67" s="3" t="n">
@@ -6245,7 +6349,11 @@
           <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M5 (model M2+M3).</t>
         </is>
       </c>
-      <c r="S67" s="4" t="inlineStr"/>
+      <c r="S67" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M3+M5'</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="110" customHeight="1">
       <c r="A68" s="3" t="n">
@@ -6423,7 +6531,11 @@
           <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M2+M3 (model M3+M1).</t>
         </is>
       </c>
-      <c r="S69" s="4" t="inlineStr"/>
+      <c r="S69" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M2+M3'</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="110" customHeight="1">
       <c r="A70" s="3" t="n">
@@ -6512,7 +6624,11 @@
           <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M3+M4 (model M4); per_kelas Y (model N).</t>
         </is>
       </c>
-      <c r="S70" s="4" t="inlineStr"/>
+      <c r="S70" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M3+M4'; akuisisi_ai='S'; per_kelas_ai='Y'</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="110" customHeight="1">
       <c r="A71" s="3" t="n">
@@ -6601,7 +6717,11 @@
           <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
         </is>
       </c>
-      <c r="S71" s="4" t="inlineStr"/>
+      <c r="S71" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M2+M3+M4'; akuisisi_ai='S'</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="110" customHeight="1">
       <c r="A72" s="3" t="n">
@@ -6690,7 +6810,11 @@
           <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: REKONSTRUKSI. Dinilai C1 dari definisi protokol; aturan Fatma untuk jenis ini belum ada, dan bila tidak dianggap C1 usul kode C5. Usul koreksi kode: akuisisi V menjadi D.</t>
         </is>
       </c>
-      <c r="S72" s="4" t="inlineStr"/>
+      <c r="S72" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: akuisisi_ai='S'</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="110" customHeight="1">
       <c r="A73" s="3" t="n">
@@ -6868,7 +6992,11 @@
           <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: STATISTIK. Dinilai C1 dari definisi protokol; aturan Fatma untuk jenis ini belum ada, dan bila tidak dianggap C1 usul kode C2. Usul koreksi kode: mekanisme M5 menjadi M1.</t>
         </is>
       </c>
-      <c r="S74" s="4" t="inlineStr"/>
+      <c r="S74" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M1'</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="110" customHeight="1">
       <c r="A75" s="3" t="n">
@@ -7046,7 +7174,11 @@
           <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
         </is>
       </c>
-      <c r="S76" s="4" t="inlineStr"/>
+      <c r="S76" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: akuisisi_ai='S'</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="110" customHeight="1">
       <c r="A77" s="3" t="n">
@@ -7135,7 +7267,11 @@
           <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
         </is>
       </c>
-      <c r="S77" s="4" t="inlineStr"/>
+      <c r="S77" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M2+M3'</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="110" customHeight="1">
       <c r="A78" s="3" t="n">
@@ -7313,7 +7449,11 @@
           <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M2+M3+M4 (model M4+M2); akuisisi V (model T).</t>
         </is>
       </c>
-      <c r="S79" s="4" t="inlineStr"/>
+      <c r="S79" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M2+M3+M4'</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="110" customHeight="1">
       <c r="A80" s="3" t="n">
@@ -7758,7 +7898,11 @@
           <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
         </is>
       </c>
-      <c r="S84" s="4" t="inlineStr"/>
+      <c r="S84" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: akuisisi_ai='S'</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="110" customHeight="1">
       <c r="A85" s="3" t="n">
@@ -8025,7 +8169,11 @@
           <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M3 (model M3+M2).</t>
         </is>
       </c>
-      <c r="S87" s="4" t="inlineStr"/>
+      <c r="S87" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M2+M3'</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="110" customHeight="1">
       <c r="A88" s="3" t="n">
@@ -8114,7 +8262,11 @@
           <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M3 (model M3+M2).</t>
         </is>
       </c>
-      <c r="S88" s="4" t="inlineStr"/>
+      <c r="S88" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M2+M3'</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="110" customHeight="1">
       <c r="A89" s="3" t="n">
@@ -9445,7 +9597,11 @@
           <t>Penilaian buta Opus 5.5, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: TIDAK_ADA. Bukan C1; usul kode C2.</t>
         </is>
       </c>
-      <c r="S103" s="4" t="inlineStr"/>
+      <c r="S103" s="4" t="inlineStr">
+        <is>
+          <t>tidak lagi C1 di sumber (kini C2); baris dipertahankan karena sudah diisi peninjau</t>
+        </is>
+      </c>
     </row>
     <row r="104" ht="110" customHeight="1">
       <c r="A104" s="3" t="n">
@@ -9534,7 +9690,11 @@
           <t>Penilaian buta Haiku 5.5 high, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M3 (model M1+M2+M3).</t>
         </is>
       </c>
-      <c r="S104" s="4" t="inlineStr"/>
+      <c r="S104" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M2+M3'</t>
+        </is>
+      </c>
     </row>
     <row r="105" ht="110" customHeight="1">
       <c r="A105" s="3" t="n">
@@ -9979,7 +10139,11 @@
           <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul koreksi kode: mekanisme M1+M2+M3 menjadi M1+M3.</t>
         </is>
       </c>
-      <c r="S109" s="4" t="inlineStr"/>
+      <c r="S109" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M2+M3'</t>
+        </is>
+      </c>
     </row>
     <row r="110" ht="110" customHeight="1">
       <c r="A110" s="3" t="n">
@@ -10068,7 +10232,11 @@
           <t>Penilaian buta Haiku 5.5 high, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M3 (model M3+M4).</t>
         </is>
       </c>
-      <c r="S110" s="4" t="inlineStr"/>
+      <c r="S110" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M3'</t>
+        </is>
+      </c>
     </row>
     <row r="111" ht="110" customHeight="1">
       <c r="A111" s="3" t="n">
@@ -10157,7 +10325,11 @@
           <t>Penilaian buta Haiku 5.5 high, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M1 (model M2+M3).</t>
         </is>
       </c>
-      <c r="S111" s="4" t="inlineStr"/>
+      <c r="S111" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M3'</t>
+        </is>
+      </c>
     </row>
     <row r="112" ht="110" customHeight="1">
       <c r="A112" s="3" t="n">
@@ -10424,7 +10596,11 @@
           <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
         </is>
       </c>
-      <c r="S114" s="4" t="inlineStr"/>
+      <c r="S114" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: akuisisi_ai='S'</t>
+        </is>
+      </c>
     </row>
     <row r="115" ht="110" customHeight="1">
       <c r="A115" s="3" t="n">
@@ -10602,7 +10778,11 @@
           <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: STATISTIK. Dinilai C1 dari definisi protokol; aturan Fatma untuk jenis ini belum ada, dan bila tidak dianggap C1 usul kode C2. Usul koreksi kode: mekanisme M0 menjadi M1; akuisisi D menjadi V.</t>
         </is>
       </c>
-      <c r="S116" s="4" t="inlineStr"/>
+      <c r="S116" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M1'</t>
+        </is>
+      </c>
     </row>
     <row r="117" ht="110" customHeight="1">
       <c r="A117" s="3" t="n">
@@ -10691,7 +10871,11 @@
           <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
         </is>
       </c>
-      <c r="S117" s="4" t="inlineStr"/>
+      <c r="S117" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M2+M3'</t>
+        </is>
+      </c>
     </row>
     <row r="118" ht="110" customHeight="1">
       <c r="A118" s="3" t="n">
@@ -11403,7 +11587,11 @@
           <t>Penilaian buta Haiku 5.5 high, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: akuisisi V (model D).</t>
         </is>
       </c>
-      <c r="S125" s="4" t="inlineStr"/>
+      <c r="S125" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: akuisisi_ai='S'</t>
+        </is>
+      </c>
     </row>
     <row r="126" ht="110" customHeight="1">
       <c r="A126" s="3" t="n">
@@ -11759,7 +11947,11 @@
           <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: TIDAK_ADA. Kasus batas: tandan dilacak antar-frame, tetapi hitungan yang dilaporkan berasal dari satu frame. Usul koreksi kode: mekanisme M2+M3 menjadi M2+M5.</t>
         </is>
       </c>
-      <c r="S129" s="4" t="inlineStr"/>
+      <c r="S129" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M3+M5'</t>
+        </is>
+      </c>
     </row>
     <row r="130" ht="110" customHeight="1">
       <c r="A130" s="3" t="n">
@@ -12026,7 +12218,11 @@
           <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
         </is>
       </c>
-      <c r="S132" s="4" t="inlineStr"/>
+      <c r="S132" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M2+M3'</t>
+        </is>
+      </c>
     </row>
     <row r="133" ht="110" customHeight="1">
       <c r="A133" s="3" t="n">
@@ -12560,7 +12756,11 @@
           <t>Penilaian buta Haiku 5.5 high, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK.</t>
         </is>
       </c>
-      <c r="S138" s="4" t="inlineStr"/>
+      <c r="S138" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: akuisisi_ai='S'</t>
+        </is>
+      </c>
     </row>
     <row r="139" ht="110" customHeight="1">
       <c r="A139" s="3" t="n">
@@ -12649,7 +12849,11 @@
           <t>Penilaian buta Haiku 5.5 high, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme DATA (model M4+M3); akuisisi D (model V).</t>
         </is>
       </c>
-      <c r="S139" s="4" t="inlineStr"/>
+      <c r="S139" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M3+M4'; akuisisi_ai='S'</t>
+        </is>
+      </c>
     </row>
     <row r="140" ht="110" customHeight="1">
       <c r="A140" s="3" t="n">
@@ -13001,7 +13205,11 @@
           <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: REKONSTRUKSI. Dinilai C1 dari definisi protokol; aturan Fatma untuk jenis ini belum ada, dan bila tidak dianggap C1 usul kode C5.</t>
         </is>
       </c>
-      <c r="S143" s="4" t="inlineStr"/>
+      <c r="S143" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: akuisisi_ai='S'</t>
+        </is>
+      </c>
     </row>
     <row r="144" ht="110" customHeight="1">
       <c r="A144" s="3" t="n">
@@ -13268,7 +13476,11 @@
           <t>Penilaian buta Haiku 5.5 high, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M3 (model M2+M3); per_kelas Y (model N).</t>
         </is>
       </c>
-      <c r="S146" s="4" t="inlineStr"/>
+      <c r="S146" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M3'; per_kelas_ai='Y'</t>
+        </is>
+      </c>
     </row>
     <row r="147" ht="110" customHeight="1">
       <c r="A147" s="3" t="n">
@@ -13446,7 +13658,11 @@
           <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
         </is>
       </c>
-      <c r="S148" s="4" t="inlineStr"/>
+      <c r="S148" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: akuisisi_ai='S'</t>
+        </is>
+      </c>
     </row>
     <row r="149" ht="110" customHeight="1">
       <c r="A149" s="3" t="n">
@@ -14514,7 +14730,11 @@
           <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
         </is>
       </c>
-      <c r="S160" s="4" t="inlineStr"/>
+      <c r="S160" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: akuisisi_ai='S'</t>
+        </is>
+      </c>
     </row>
     <row r="161" ht="110" customHeight="1">
       <c r="A161" s="3" t="n">
@@ -14781,7 +15001,11 @@
           <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: REKONSTRUKSI. Dinilai C1 dari definisi protokol; aturan Fatma untuk jenis ini belum ada, dan bila tidak dianggap C1 usul kode C2. Usul koreksi kode: akuisisi V menjadi D.</t>
         </is>
       </c>
-      <c r="S163" s="4" t="inlineStr"/>
+      <c r="S163" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M4'; akuisisi_ai='D'</t>
+        </is>
+      </c>
     </row>
     <row r="164" ht="110" customHeight="1">
       <c r="A164" s="3" t="n">
@@ -14870,7 +15094,11 @@
           <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK.</t>
         </is>
       </c>
-      <c r="S164" s="4" t="inlineStr"/>
+      <c r="S164" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: akuisisi_ai='S'</t>
+        </is>
+      </c>
     </row>
     <row r="165" ht="110" customHeight="1">
       <c r="A165" s="3" t="n">
@@ -15485,7 +15713,11 @@
           <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
         </is>
       </c>
-      <c r="S171" s="4" t="inlineStr"/>
+      <c r="S171" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: akuisisi_ai='S'</t>
+        </is>
+      </c>
     </row>
     <row r="172" ht="110" customHeight="1">
       <c r="A172" s="3" t="n">
@@ -15574,7 +15806,11 @@
           <t>Penilaian buta Haiku 5.5 high, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M3+M4 (model M2+M3).</t>
         </is>
       </c>
-      <c r="S172" s="4" t="inlineStr"/>
+      <c r="S172" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M3+M4'</t>
+        </is>
+      </c>
     </row>
     <row r="173" ht="110" customHeight="1">
       <c r="A173" s="3" t="n">
@@ -15752,7 +15988,11 @@
           <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
         </is>
       </c>
-      <c r="S174" s="4" t="inlineStr"/>
+      <c r="S174" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: akuisisi_ai='S'</t>
+        </is>
+      </c>
     </row>
     <row r="175" ht="110" customHeight="1">
       <c r="A175" s="3" t="n">
@@ -15841,7 +16081,11 @@
           <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
         </is>
       </c>
-      <c r="S175" s="4" t="inlineStr"/>
+      <c r="S175" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: akuisisi_ai='S'</t>
+        </is>
+      </c>
     </row>
     <row r="176" ht="110" customHeight="1">
       <c r="A176" s="3" t="n">
@@ -16286,7 +16530,11 @@
           <t>Penilaian buta Haiku 5.5 high, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: akuisisi V (model D).</t>
         </is>
       </c>
-      <c r="S180" s="4" t="inlineStr"/>
+      <c r="S180" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M3+M4'; akuisisi_ai='S'</t>
+        </is>
+      </c>
     </row>
     <row r="181" ht="110" customHeight="1">
       <c r="A181" s="3" t="n">
@@ -16553,7 +16801,11 @@
           <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul koreksi kode: mekanisme M1 menjadi M1+M4.</t>
         </is>
       </c>
-      <c r="S183" s="4" t="inlineStr"/>
+      <c r="S183" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M4'</t>
+        </is>
+      </c>
     </row>
     <row r="184" ht="110" customHeight="1">
       <c r="A184" s="3" t="n">
@@ -16642,7 +16894,11 @@
           <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
         </is>
       </c>
-      <c r="S184" s="4" t="inlineStr"/>
+      <c r="S184" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M4'</t>
+        </is>
+      </c>
     </row>
     <row r="185" ht="110" customHeight="1">
       <c r="A185" s="3" t="n">
@@ -16731,7 +16987,11 @@
           <t>Penilaian buta Haiku 5.5 high, 11 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: LACAK. Usul kode: mekanisme M2 (model M1); akuisisi T (model D).</t>
         </is>
       </c>
-      <c r="S185" s="4" t="inlineStr"/>
+      <c r="S185" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M4'; akuisisi_ai='V'</t>
+        </is>
+      </c>
     </row>
     <row r="186" ht="110" customHeight="1">
       <c r="A186" s="3" t="n">
@@ -17083,7 +17343,11 @@
           <t>Diisi 11 Oktober 2026 atas instruksi peninjau berdasarkan pemeriksaan Haiku (hasil-kerja-ai/menunggu-acc/cek-2); belum dibaca peninjau</t>
         </is>
       </c>
-      <c r="S189" s="4" t="inlineStr"/>
+      <c r="S189" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: mekanisme_ai='M4'; akuisisi_ai='S'</t>
+        </is>
+      </c>
     </row>
     <row r="190" ht="110" customHeight="1">
       <c r="A190" s="3" t="n">
@@ -17427,7 +17691,11 @@
           <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: TIDAK_ADA. Bukan C1; usul kode C2.</t>
         </is>
       </c>
-      <c r="S193" s="4" t="inlineStr"/>
+      <c r="S193" s="4" t="inlineStr">
+        <is>
+          <t>tidak lagi C1 di sumber (kini C2); baris dipertahankan karena sudah diisi peninjau</t>
+        </is>
+      </c>
     </row>
     <row r="194" ht="110" customHeight="1">
       <c r="A194" s="3" t="n">
@@ -17512,7 +17780,11 @@
           <t>Penilaian buta Opus 5.5 dan verifikasi ulang oleh agen Opus 5.5 kedua, 12 Oktober 2026, diisi atas instruksi peninjau; belum dibaca peninjau. Jenis penggabungan: REKONSTRUKSI. Dinilai C1 dari definisi protokol; aturan Fatma untuk jenis ini belum ada, dan bila tidak dianggap C1 usul kode C5.</t>
         </is>
       </c>
-      <c r="S194" s="4" t="inlineStr"/>
+      <c r="S194" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: akuisisi_ai='S'</t>
+        </is>
+      </c>
     </row>
     <row r="195" ht="110" customHeight="1">
       <c r="A195" s="3" t="n">
@@ -17775,7 +18047,11 @@
           <t>Diisi 18 Oktober 2026 dari ajudikasi Cek 1 (dua pembaca buta Haiku 5.5 + penengah, diperiksa agen utama; diserahkan peninjau), cek-1-sampel-buta/ajudikasi/ajudikasi_cek1.csv. Isian model, bukan bacaan peninjau. Model 3D SfM/MVS dari video harian; aturan rekonstruksi 3D (TUGAS 1.1).</t>
         </is>
       </c>
-      <c r="S197" s="4" t="inlineStr"/>
+      <c r="S197" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: akuisisi_ai='S'</t>
+        </is>
+      </c>
     </row>
     <row r="198" ht="110" customHeight="1">
       <c r="A198" s="3" t="n">
@@ -17860,15 +18136,461 @@
           <t>Diisi 18 Oktober 2026 dari ajudikasi Cek 1 (dua pembaca buta Haiku 5.5 + penengah, diperiksa agen utama; diserahkan peninjau), cek-1-sampel-buta/ajudikasi/ajudikasi_cek1.csv. Isian model, bukan bacaan peninjau. Hitungan dengan pelacakan centroid antar-frame.</t>
         </is>
       </c>
-      <c r="S198" s="4" t="inlineStr"/>
+      <c r="S198" s="4" t="inlineStr">
+        <is>
+          <t>sumber kini: per_kelas_ai='Y'</t>
+        </is>
+      </c>
+    </row>
+    <row r="199" ht="110" customHeight="1">
+      <c r="A199" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="B199" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="C199" s="3" t="inlineStr">
+        <is>
+          <t>yokin20263d</t>
+        </is>
+      </c>
+      <c r="D199" s="3" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E199" s="4" t="inlineStr">
+        <is>
+          <t>3D reconstruction and segmentation of grape bunches for robotic berry thinning</t>
+        </is>
+      </c>
+      <c r="F199" s="3" t="inlineStr">
+        <is>
+          <t>10.1016/j.compag.2026.111898</t>
+        </is>
+      </c>
+      <c r="G199" s="4" t="inlineStr">
+        <is>
+          <t>• End-to-end pipeline from neural reconstruction to physical grape berry manipulation. • Efficient point clouds generation using NeRF and the metric scale derived directly from robot kinematics. • RANSAC sphere fitting achieves 92.1% berry detection precision without annotated training data. • Stem-aligned 6-DoF pose optimization improves end-to-end grip success by 17.2%. Table grape thinning requires selective removal of 20–40% of berries from dense clusters. In practice, workers decide which berries to remove by considering both the approximate berry count and local 3D spatial characteristics such as crowding and relative positioning. Automating this task is challenging because conventional 2D image-based approaches suffer from occlusion-related counting errors and lack explicit 3D spatial information necessary for reliable manipulation. We propose a robot-integrated vision pipeline that reconstructs grape bunch structure from posed multi-view RGB images. Neural Radiance Fields (NeRF) is used to learn a volumetric scene representation, from which a dense, low-noise point cloud is extracted via depth back-projection, and RANSAC-based geometric fitting models individual berries and stems, enabling berry-level segmentation and orientation estimation for manipulation planning. The perception pipeline uses an eye-in-hand RealSense D405 camera mounted on a Fanuc CRX-5iA collaborative robot. Camera poses are derived from the robot kinematic chain, allowing the reconstructed point cloud and detected berry centers to be expressed directly in the metric robot base frame without external scale recovery. In robot-mounted RealSense D405 experiments on 10 grape bunches, RANSAC sphere fitting achieved a counting MAE of 0.50 berries, RMSE of 0.71 berries, and mean center localization error of 2.71 mm. On a 52-bunch benchmark, RANSAC sphere fitting outperforms the learning-based SoftGroup++ method for 3D berry instance segmentation (92.1% vs 82.8% average precision) without requiring annotated training data. In 35 manipulation trials, the system achieved an 85.7% pre-grasp reachability rate and an 83.3% conditional target success rate demonstrating an end-to-end pipeline from neural reconstruction to manipulation-ready berry poses.</t>
+        </is>
+      </c>
+      <c r="H199" s="3" t="inlineStr">
+        <is>
+          <t>abstrak</t>
+        </is>
+      </c>
+      <c r="I199" s="3" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="J199" s="3" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="K199" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L199" s="4" t="inlineStr">
+        <is>
+          <t>tandan anggur, robot penjarang; NeRF dari citra multipandang berpose, butir disegmentasi dan dicacah di awan titik</t>
+        </is>
+      </c>
+      <c r="M199" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N199" s="3" t="inlineStr"/>
+      <c r="O199" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P199" s="5" t="inlineStr"/>
+      <c r="Q199" s="5" t="inlineStr"/>
+      <c r="R199" s="6" t="inlineStr"/>
+      <c r="S199" s="4" t="inlineStr"/>
+    </row>
+    <row r="200" ht="110" customHeight="1">
+      <c r="A200" s="3" t="n">
+        <v>201</v>
+      </c>
+      <c r="B200" s="3" t="n">
+        <v>467</v>
+      </c>
+      <c r="C200" s="3" t="inlineStr">
+        <is>
+          <t>daud2023detection</t>
+        </is>
+      </c>
+      <c r="D200" s="3" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="E200" s="4" t="inlineStr">
+        <is>
+          <t>Detection of Oil Palm Tree and Loose Fruitlets for Fresh Fruit Bunch's Ready-to-Harvest Prediction via Deep Learning Approach</t>
+        </is>
+      </c>
+      <c r="F200" s="3" t="inlineStr"/>
+      <c r="G200" s="4" t="inlineStr"/>
+      <c r="H200" s="3" t="inlineStr">
+        <is>
+          <t>abstrak</t>
+        </is>
+      </c>
+      <c r="I200" s="3" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="J200" s="3" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="K200" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L200" s="4" t="inlineStr">
+        <is>
+          <t>brondolan sawit; pelacakan pohon antar-frame dan hitungan per pohon dari frekuensi terbanyak selama n frame; prediksi siap panen</t>
+        </is>
+      </c>
+      <c r="M200" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N200" s="3" t="inlineStr">
+        <is>
+          <t>literature/scopus-2026-09/teks/daud2023detection.txt</t>
+        </is>
+      </c>
+      <c r="O200" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P200" s="5" t="inlineStr"/>
+      <c r="Q200" s="5" t="inlineStr"/>
+      <c r="R200" s="6" t="inlineStr"/>
+      <c r="S200" s="4" t="inlineStr"/>
+    </row>
+    <row r="201" ht="110" customHeight="1">
+      <c r="A201" s="3" t="n">
+        <v>202</v>
+      </c>
+      <c r="B201" s="3" t="n">
+        <v>434</v>
+      </c>
+      <c r="C201" s="3" t="inlineStr">
+        <is>
+          <t>shiddiq2023counting</t>
+        </is>
+      </c>
+      <c r="D201" s="3" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="E201" s="4" t="inlineStr">
+        <is>
+          <t>COUNTING OF OIL PALM FRESH FRUIT BUNCHES USING COMPUTER VISION</t>
+        </is>
+      </c>
+      <c r="F201" s="3" t="inlineStr">
+        <is>
+          <t>10.21894/jopr.2022.0029</t>
+        </is>
+      </c>
+      <c r="G201" s="4" t="inlineStr">
+        <is>
+          <t>Oil palm fresh fruit bunches (FFB) are the sources of crude palm oil (CPO). CPO is one of the largest export commodities for Indonesia and Malaysia. Automation or mechanisation in CPO processes is crucial to saving time, labour, and cost. This study used the computer vision method to count moving oil palm FFB using video frames. It is possible to implement this counting method in the oil palm FFB sorting and grading stage to estimate the CPO mill capacity. Video recordings used an RGB camera with a frame rate of 20 FPS for 117 oil palm FFB of Tenera varieties. The counting program consisted of two parts, a detector and a tracker. The detector algorithm was self-developed by adding a colour feature, converting the RGB images of oil palm FFB to HSV colour space. The counting results were validated using the confusion matrix method. The results showed that the counting accuracy could reach 100.00%. However, the counting accuracy depends on the colour of the FFB and room light intensity. The confusion matrix validation resulted in average counting accuracy of 79.35% for 10 videos. The results showed the potential use of computer vision in counting moving oil palm FFB.</t>
+        </is>
+      </c>
+      <c r="H201" s="3" t="inlineStr">
+        <is>
+          <t>abstrak</t>
+        </is>
+      </c>
+      <c r="I201" s="3" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="J201" s="3" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="K201" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L201" s="4" t="inlineStr">
+        <is>
+          <t>TBS sawit bergerak di konveyor; detektor + pelacak centroid antar-frame; akurasi hitung sampai 100%</t>
+        </is>
+      </c>
+      <c r="M201" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N201" s="3" t="inlineStr">
+        <is>
+          <t>literature/scopus-2026-09/teks/shiddiq2023counting.txt</t>
+        </is>
+      </c>
+      <c r="O201" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P201" s="5" t="inlineStr"/>
+      <c r="Q201" s="5" t="inlineStr"/>
+      <c r="R201" s="6" t="inlineStr"/>
+      <c r="S201" s="4" t="inlineStr"/>
+    </row>
+    <row r="202" ht="110" customHeight="1">
+      <c r="A202" s="3" t="n">
+        <v>203</v>
+      </c>
+      <c r="B202" s="3" t="n">
+        <v>551</v>
+      </c>
+      <c r="C202" s="3" t="inlineStr">
+        <is>
+          <t>daud2022loose</t>
+        </is>
+      </c>
+      <c r="D202" s="3" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="E202" s="4" t="inlineStr">
+        <is>
+          <t>Loose Fruitlet and Fresh Fruit Bunch Detection for Palm Oil Harvest Management</t>
+        </is>
+      </c>
+      <c r="F202" s="3" t="inlineStr">
+        <is>
+          <t>10.1109/iotais56727.2022.9975972</t>
+        </is>
+      </c>
+      <c r="G202" s="4" t="inlineStr">
+        <is>
+          <t>The palm oil industry can be considered one of the crucial industries, especially in Asian countries like Malaysia and Indonesia. The production flow is depending on the efficiency of the palm oil harvest management. The management during harvest time includes collecting and counting the fresh fruit bunch (FFB) and loose fruitlet (LF) production. Thus, in this paper, we proposed a method that able to detect and count the FFB and LF production automatically. The as-proposed method consisted of two parts: (a) fruitlet detection using an image processing prior to harvest and (b) palm oil tree, FFB, and grabber detection using the Faster R-CNN algorithm during harvest time. During the pre-harvest, the number of fruitlets can be determined through the status of the tree either by ready-to-harvest (RTH) or not ready-to-harvest (NRTH). If the status was RTH, the system performed tree detection for tagging purposes. When they started to harvest, the detection system would detect the FFB and grabber. It would then track the grabber until overlaps with the FFB location. Then, the system would add the FFB to the count module. It means the FFB had been taken to the truck. The as-proposed system achieved the detection accuracy of 96.5% for FFB, 99.2% for grabber, and 97.2% for tree.</t>
+        </is>
+      </c>
+      <c r="H202" s="3" t="inlineStr">
+        <is>
+          <t>abstrak</t>
+        </is>
+      </c>
+      <c r="I202" s="3" t="inlineStr">
+        <is>
+          <t>M0+M3</t>
+        </is>
+      </c>
+      <c r="J202" s="3" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="K202" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L202" s="4" t="inlineStr">
+        <is>
+          <t>brondolan sawit di bawah pohon; pelacakan pohon antar-frame, hitungan per pohon dari modus hitungan per frame; hitungan TBS terkumpul per frame</t>
+        </is>
+      </c>
+      <c r="M202" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N202" s="3" t="inlineStr">
+        <is>
+          <t>literature/scopus-2026-09/teks/daud2022loose.txt</t>
+        </is>
+      </c>
+      <c r="O202" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P202" s="5" t="inlineStr"/>
+      <c r="Q202" s="5" t="inlineStr"/>
+      <c r="R202" s="6" t="inlineStr"/>
+      <c r="S202" s="4" t="inlineStr"/>
+    </row>
+    <row r="203" ht="110" customHeight="1">
+      <c r="A203" s="3" t="n">
+        <v>204</v>
+      </c>
+      <c r="B203" s="3" t="n">
+        <v>625</v>
+      </c>
+      <c r="C203" s="3" t="inlineStr">
+        <is>
+          <t>aji2021automatic</t>
+        </is>
+      </c>
+      <c r="D203" s="3" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="E203" s="4" t="inlineStr">
+        <is>
+          <t>Automatic Oil Palm Unstripped Bunch (USB) Counting System based on Faster RCNN and Object Tracking</t>
+        </is>
+      </c>
+      <c r="F203" s="3" t="inlineStr">
+        <is>
+          <t>10.1109/ic2se52832.2021.9792068</t>
+        </is>
+      </c>
+      <c r="G203" s="4" t="inlineStr">
+        <is>
+          <t>USB Palm Oil Counting (Unstripped Bunch) is important in oil palm processing mills. Information on the number of USBs is essential because it shows the level of efficiency of the palm oil processing plant. Due to its complexity, palm oil mills rely solely on manual calculations, which is inefficient workforce waste. Challenging aspects such as partial occlusion, overlap, and even different perspectives limit the use of traditional computer vision techniques. In recent years, deep learning has become increasingly popular for computer vision applications due to its superior performance over conventional methods. This paper proposes a deep learning solution to solve USB computing problems in palm oil mills. Our proposed automated USB counter system consists of an object detector built on the RCNN Faster architecture and an object tracker made in the euclidean distance. Our proposed system identifies and counts USBs with an average accuracy of 71.5% in testing.</t>
+        </is>
+      </c>
+      <c r="H203" s="3" t="inlineStr">
+        <is>
+          <t>abstrak</t>
+        </is>
+      </c>
+      <c r="I203" s="3" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="J203" s="3" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="K203" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L203" s="4" t="inlineStr">
+        <is>
+          <t>tandan tak terpipil (USB) sawit di pabrik; Faster R-CNN + pelacakan centroid antar-frame; hitungan dievaluasi</t>
+        </is>
+      </c>
+      <c r="M203" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N203" s="3" t="inlineStr">
+        <is>
+          <t>literature/scopus-2026-09/teks/aji2021automatic.txt</t>
+        </is>
+      </c>
+      <c r="O203" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P203" s="5" t="inlineStr"/>
+      <c r="Q203" s="5" t="inlineStr"/>
+      <c r="R203" s="6" t="inlineStr"/>
+      <c r="S203" s="4" t="inlineStr"/>
+    </row>
+    <row r="204" ht="110" customHeight="1">
+      <c r="A204" s="3" t="n">
+        <v>205</v>
+      </c>
+      <c r="B204" s="3" t="n">
+        <v>2483</v>
+      </c>
+      <c r="C204" s="3" t="inlineStr">
+        <is>
+          <t>kassim2012oil</t>
+        </is>
+      </c>
+      <c r="D204" s="3" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="E204" s="4" t="inlineStr">
+        <is>
+          <t>Oil palm fresh fruit bunches (FFB) growth determination system to support harvesting operation</t>
+        </is>
+      </c>
+      <c r="F204" s="3" t="inlineStr"/>
+      <c r="G204" s="4" t="inlineStr"/>
+      <c r="H204" s="3" t="inlineStr">
+        <is>
+          <t>abstrak</t>
+        </is>
+      </c>
+      <c r="I204" s="3" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="J204" s="3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="K204" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L204" s="4" t="inlineStr">
+        <is>
+          <t>TBS sawit; 809 tandan diberi tag dan dipantau berulang dari antesis sampai panen (sekitar 30.000 citra); umur dan tanggal panen per tandan</t>
+        </is>
+      </c>
+      <c r="M204" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N204" s="3" t="inlineStr">
+        <is>
+          <t>literature/scopus-2026-09/teks/kassim2012oil.txt</t>
+        </is>
+      </c>
+      <c r="O204" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P204" s="5" t="inlineStr"/>
+      <c r="Q204" s="5" t="inlineStr"/>
+      <c r="R204" s="6" t="inlineStr"/>
+      <c r="S204" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S198"/>
+  <autoFilter ref="A1:S204"/>
   <dataValidations count="2">
-    <dataValidation sqref="P2:P398" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak sah" error="Pilih salah satu: Y,N" type="list">
+    <dataValidation sqref="P2:P404" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak sah" error="Pilih salah satu: Y,N" type="list">
       <formula1>"Y,N"</formula1>
     </dataValidation>
-    <dataValidation sqref="Q2:Q398" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak sah" error="Pilih salah satu: Y,N" type="list">
+    <dataValidation sqref="Q2:Q404" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak sah" error="Pilih salah satu: Y,N" type="list">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>